<commit_message>
feat: refactor icon generation workflow
</commit_message>
<xml_diff>
--- a/outputs/2026-08-20-development-plan/IconGen-前后端原子级开发计划.xlsx
+++ b/outputs/2026-08-20-development-plan/IconGen-前后端原子级开发计划.xlsx
@@ -2,9 +2,9 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="阶段概览" sheetId="1" r:id="Rec500e56b742436e"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="前端开发计划" sheetId="2" r:id="R2426ffeae60048d7"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="后端开发计划" sheetId="3" r:id="R9dabeabeaad344da"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="阶段概览" sheetId="1" r:id="R760c11cde2174b81"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="前端开发计划" sheetId="2" r:id="R7b1e4804122f4fa2"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="后端开发计划" sheetId="3" r:id="R9c89e8b0ce424125"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -456,7 +456,7 @@
     </x:row>
     <x:row r="2">
       <x:c r="A2" t="str">
-        <x:v>更新时间：2026-08-21；状态以代码、PRD 与本工作簿一致性验收为准</x:v>
+        <x:v>更新时间：2026-08-22；创建页已重构为图标设计风格：5个预设 + 3组微调；颜色、背景形状与尺寸独立；请求和Skill统一使用style字段</x:v>
       </x:c>
     </x:row>
     <x:row r="3" ht="34" customHeight="1">
@@ -503,15 +503,15 @@
       </x:c>
       <x:c r="E4" s="14" t="n">
         <x:f>COUNTIF('前端开发计划'!K4:K260,"已完成")</x:f>
-        <x:v>56</x:v>
+        <x:v>139</x:v>
       </x:c>
       <x:c r="F4" s="14" t="n">
         <x:f>D4-E4</x:f>
-        <x:v>201</x:v>
+        <x:v>118</x:v>
       </x:c>
       <x:c r="G4" s="15" t="n">
         <x:f>E4/D4</x:f>
-        <x:v>0.2178988326848249</x:v>
+        <x:v>0.5408560311284046</x:v>
       </x:c>
       <x:c r="H4" s="14" t="str">
         <x:v>一个动作、一个交付物、一个独立验收结果</x:v>
@@ -535,15 +535,15 @@
       </x:c>
       <x:c r="E5" s="14" t="n">
         <x:f>COUNTIF('后端开发计划'!K4:K294,"已完成")</x:f>
-        <x:v>67</x:v>
+        <x:v>108</x:v>
       </x:c>
       <x:c r="F5" s="14" t="n">
         <x:f>D5-E5</x:f>
-        <x:v>224</x:v>
+        <x:v>183</x:v>
       </x:c>
       <x:c r="G5" s="15" t="n">
         <x:f>E5/D5</x:f>
-        <x:v>0.23024054982817868</x:v>
+        <x:v>0.3711340206185567</x:v>
       </x:c>
       <x:c r="H5" s="14" t="str">
         <x:v>一个动作、一个交付物、一个独立验收结果</x:v>
@@ -5457,25 +5457,25 @@
         <x:v>前端</x:v>
       </x:c>
       <x:c r="G89" s="13" t="str">
-        <x:v>建立创建页主体编辑区路由与页面边界</x:v>
+        <x:v>精简图标主体输入反馈</x:v>
       </x:c>
       <x:c r="H89" s="13" t="str">
-        <x:v>创建页主体编辑区路由、页面组件和Metadata</x:v>
+        <x:v>移除“已识别 N 个图标主体”动态提示</x:v>
       </x:c>
       <x:c r="I89" s="13" t="str">
-        <x:v>直接访问路由可渲染；未授权跳转符合PRD；无运行时错误</x:v>
+        <x:v>保留输入引导、主体解析和提交校验；页面不展示主体计数文案</x:v>
       </x:c>
       <x:c r="J89" s="13" t="str">
         <x:v>—</x:v>
       </x:c>
       <x:c r="K89" s="13" t="str">
-        <x:v>待完成</x:v>
+        <x:v>已完成</x:v>
       </x:c>
       <x:c r="L89" s="13" t="str">
         <x:v>08-22～08-24</x:v>
       </x:c>
       <x:c r="M89" s="13" t="str">
-        <x:v>—</x:v>
+        <x:v>2026-08-22</x:v>
       </x:c>
       <x:c r="N89" s="13" t="str">
         <x:v>job/subject/variant/asset均为UUID；创建请求带idempotency_key；记录设置/Skill/模型版本</x:v>
@@ -5513,25 +5513,25 @@
         <x:v>前端</x:v>
       </x:c>
       <x:c r="G90" s="13" t="str">
-        <x:v>定义创建页主体编辑区页面状态模型</x:v>
+        <x:v>定义批量描述输入状态</x:v>
       </x:c>
       <x:c r="H90" s="13" t="str">
-        <x:v>页面状态类型与初始化逻辑</x:v>
+        <x:v>原始文本、解析主体和校验错误</x:v>
       </x:c>
       <x:c r="I90" s="13" t="str">
-        <x:v>每个状态只有一个含义；刷新后可恢复服务端状态</x:v>
+        <x:v>输入变化后解析结果同步更新</x:v>
       </x:c>
       <x:c r="J90" s="13" t="str">
         <x:v>FE-CREATE-SUBJECT-01</x:v>
       </x:c>
       <x:c r="K90" s="13" t="str">
-        <x:v>待完成</x:v>
+        <x:v>已完成</x:v>
       </x:c>
       <x:c r="L90" s="13" t="str">
         <x:v>08-22～08-24</x:v>
       </x:c>
       <x:c r="M90" s="13" t="str">
-        <x:v>—</x:v>
+        <x:v>2026-08-21</x:v>
       </x:c>
       <x:c r="N90" s="13" t="str">
         <x:v>job/subject/variant/asset均为UUID；创建请求带idempotency_key；记录设置/Skill/模型版本</x:v>
@@ -5569,25 +5569,25 @@
         <x:v>前端</x:v>
       </x:c>
       <x:c r="G91" s="13" t="str">
-        <x:v>实现新增主体</x:v>
+        <x:v>实现单一多行输入框</x:v>
       </x:c>
       <x:c r="H91" s="13" t="str">
-        <x:v>新增空主体行</x:v>
+        <x:v>一个textarea承载全部图标需求</x:v>
       </x:c>
       <x:c r="I91" s="13" t="str">
-        <x:v>最多20个；新增后焦点正确</x:v>
+        <x:v>支持中文和英文内容并保留换行</x:v>
       </x:c>
       <x:c r="J91" s="13" t="str">
         <x:v>—</x:v>
       </x:c>
       <x:c r="K91" s="13" t="str">
-        <x:v>待完成</x:v>
+        <x:v>已完成</x:v>
       </x:c>
       <x:c r="L91" s="13" t="str">
         <x:v>08-22～08-24</x:v>
       </x:c>
       <x:c r="M91" s="13" t="str">
-        <x:v>—</x:v>
+        <x:v>2026-08-21</x:v>
       </x:c>
       <x:c r="N91" s="13" t="str">
         <x:v>job/subject/variant/asset均为UUID；创建请求带idempotency_key；记录设置/Skill/模型版本</x:v>
@@ -5625,25 +5625,25 @@
         <x:v>前端</x:v>
       </x:c>
       <x:c r="G92" s="13" t="str">
-        <x:v>实现删除主体</x:v>
+        <x:v>按行解析多个主体</x:v>
       </x:c>
       <x:c r="H92" s="13" t="str">
-        <x:v>删除指定主体</x:v>
+        <x:v>每个非空行生成一个subject</x:v>
       </x:c>
       <x:c r="I92" s="13" t="str">
-        <x:v>至少保留1个；误删前确认策略明确</x:v>
+        <x:v>空行被忽略且不设置20个主体上限</x:v>
       </x:c>
       <x:c r="J92" s="13" t="str">
         <x:v>—</x:v>
       </x:c>
       <x:c r="K92" s="13" t="str">
-        <x:v>待完成</x:v>
+        <x:v>已完成</x:v>
       </x:c>
       <x:c r="L92" s="13" t="str">
         <x:v>08-22～08-24</x:v>
       </x:c>
       <x:c r="M92" s="13" t="str">
-        <x:v>—</x:v>
+        <x:v>2026-08-21</x:v>
       </x:c>
       <x:c r="N92" s="13" t="str">
         <x:v>job/subject/variant/asset均为UUID；创建请求带idempotency_key；记录设置/Skill/模型版本</x:v>
@@ -5681,25 +5681,25 @@
         <x:v>前端</x:v>
       </x:c>
       <x:c r="G93" s="13" t="str">
-        <x:v>实现主体排序</x:v>
+        <x:v>解析名称与描述</x:v>
       </x:c>
       <x:c r="H93" s="13" t="str">
-        <x:v>上移/下移或拖拽</x:v>
+        <x:v>支持“名称：功能与视觉含义”格式</x:v>
       </x:c>
       <x:c r="I93" s="13" t="str">
-        <x:v>clientId保持稳定</x:v>
+        <x:v>冒号前为名称、冒号后为描述；无冒号时整行可提交</x:v>
       </x:c>
       <x:c r="J93" s="13" t="str">
         <x:v>—</x:v>
       </x:c>
       <x:c r="K93" s="13" t="str">
-        <x:v>待完成</x:v>
+        <x:v>已完成</x:v>
       </x:c>
       <x:c r="L93" s="13" t="str">
         <x:v>08-22～08-24</x:v>
       </x:c>
       <x:c r="M93" s="13" t="str">
-        <x:v>—</x:v>
+        <x:v>2026-08-21</x:v>
       </x:c>
       <x:c r="N93" s="13" t="str">
         <x:v>job/subject/variant/asset均为UUID；创建请求带idempotency_key；记录设置/Skill/模型版本</x:v>
@@ -5737,25 +5737,25 @@
         <x:v>前端</x:v>
       </x:c>
       <x:c r="G94" s="13" t="str">
-        <x:v>实现批量粘贴解析</x:v>
+        <x:v>展示识别主体数量</x:v>
       </x:c>
       <x:c r="H94" s="13" t="str">
-        <x:v>逐行转换为主体</x:v>
+        <x:v>实时主体计数提示</x:v>
       </x:c>
       <x:c r="I94" s="13" t="str">
-        <x:v>空行去除；超限明确提示</x:v>
+        <x:v>计数与最终subjects数组一致</x:v>
       </x:c>
       <x:c r="J94" s="13" t="str">
         <x:v>—</x:v>
       </x:c>
       <x:c r="K94" s="13" t="str">
-        <x:v>待完成</x:v>
+        <x:v>已完成</x:v>
       </x:c>
       <x:c r="L94" s="13" t="str">
         <x:v>08-22～08-24</x:v>
       </x:c>
       <x:c r="M94" s="13" t="str">
-        <x:v>—</x:v>
+        <x:v>2026-08-21</x:v>
       </x:c>
       <x:c r="N94" s="13" t="str">
         <x:v>job/subject/variant/asset均为UUID；创建请求带idempotency_key；记录设置/Skill/模型版本</x:v>
@@ -5793,25 +5793,25 @@
         <x:v>前端</x:v>
       </x:c>
       <x:c r="G95" s="13" t="str">
-        <x:v>实现名称和描述校验</x:v>
+        <x:v>校验批量主体内容</x:v>
       </x:c>
       <x:c r="H95" s="13" t="str">
-        <x:v>name 1–40、description 2–300</x:v>
+        <x:v>至少1项、名称1–40、描述2–300</x:v>
       </x:c>
       <x:c r="I95" s="13" t="str">
-        <x:v>逐主体定位错误</x:v>
+        <x:v>错误阻止提交并保留输入</x:v>
       </x:c>
       <x:c r="J95" s="13" t="str">
         <x:v>—</x:v>
       </x:c>
       <x:c r="K95" s="13" t="str">
-        <x:v>待完成</x:v>
+        <x:v>已完成</x:v>
       </x:c>
       <x:c r="L95" s="13" t="str">
         <x:v>08-22～08-24</x:v>
       </x:c>
       <x:c r="M95" s="13" t="str">
-        <x:v>—</x:v>
+        <x:v>2026-08-21</x:v>
       </x:c>
       <x:c r="N95" s="13" t="str">
         <x:v>job/subject/variant/asset均为UUID；创建请求带idempotency_key；记录设置/Skill/模型版本</x:v>
@@ -5852,7 +5852,7 @@
         <x:v>实现本地草稿保存</x:v>
       </x:c>
       <x:c r="H96" s="13" t="str">
-        <x:v>版本化草稿结构</x:v>
+        <x:v>版本化原始文本草稿</x:v>
       </x:c>
       <x:c r="I96" s="13" t="str">
         <x:v>刷新恢复；提交成功后按规则清理</x:v>
@@ -5905,25 +5905,25 @@
         <x:v>前端</x:v>
       </x:c>
       <x:c r="G97" s="13" t="str">
-        <x:v>接入创建页主体编辑区服务端接口</x:v>
+        <x:v>接入生成任务请求Schema</x:v>
       </x:c>
       <x:c r="H97" s="13" t="str">
-        <x:v>本地草稿+generation schema客户端适配器</x:v>
+        <x:v>批量文本解析为subjects数组</x:v>
       </x:c>
       <x:c r="I97" s="13" t="str">
-        <x:v>请求字段与共享Schema一致；不在组件内拼装不受控请求</x:v>
+        <x:v>clientId唯一且请求不含主体数量上限字段</x:v>
       </x:c>
       <x:c r="J97" s="13" t="str">
         <x:v>FE-CREATE-SUBJECT-02</x:v>
       </x:c>
       <x:c r="K97" s="13" t="str">
-        <x:v>待完成</x:v>
+        <x:v>已完成</x:v>
       </x:c>
       <x:c r="L97" s="13" t="str">
         <x:v>08-22～08-24</x:v>
       </x:c>
       <x:c r="M97" s="13" t="str">
-        <x:v>—</x:v>
+        <x:v>2026-08-21</x:v>
       </x:c>
       <x:c r="N97" s="13" t="str">
         <x:v>job/subject/variant/asset均为UUID；创建请求带idempotency_key；记录设置/Skill/模型版本</x:v>
@@ -5961,25 +5961,25 @@
         <x:v>前端</x:v>
       </x:c>
       <x:c r="G98" s="13" t="str">
-        <x:v>实现创建页主体编辑区加载状态</x:v>
+        <x:v>实现设置加载状态</x:v>
       </x:c>
       <x:c r="H98" s="13" t="str">
-        <x:v>骨架屏或进度反馈</x:v>
+        <x:v>设置接口加载反馈</x:v>
       </x:c>
       <x:c r="I98" s="13" t="str">
-        <x:v>请求期间有可感知反馈；重复操作被禁用</x:v>
+        <x:v>加载期间禁用生成提交</x:v>
       </x:c>
       <x:c r="J98" s="13" t="str">
         <x:v>FE-CREATE-SUBJECT-02</x:v>
       </x:c>
       <x:c r="K98" s="13" t="str">
-        <x:v>待完成</x:v>
+        <x:v>已完成</x:v>
       </x:c>
       <x:c r="L98" s="13" t="str">
         <x:v>08-22～08-24</x:v>
       </x:c>
       <x:c r="M98" s="13" t="str">
-        <x:v>—</x:v>
+        <x:v>2026-08-21</x:v>
       </x:c>
       <x:c r="N98" s="13" t="str">
         <x:v>job/subject/variant/asset均为UUID；创建请求带idempotency_key；记录设置/Skill/模型版本</x:v>
@@ -6017,25 +6017,25 @@
         <x:v>前端</x:v>
       </x:c>
       <x:c r="G99" s="13" t="str">
-        <x:v>实现创建页主体编辑区错误映射</x:v>
+        <x:v>实现批量输入错误提示</x:v>
       </x:c>
       <x:c r="H99" s="13" t="str">
-        <x:v>稳定错误码到双语用户文案的映射</x:v>
+        <x:v>双语校验和服务端错误提示</x:v>
       </x:c>
       <x:c r="I99" s="13" t="str">
-        <x:v>业务错误可恢复；未知错误不泄露内部信息</x:v>
+        <x:v>未知错误不泄露内部信息</x:v>
       </x:c>
       <x:c r="J99" s="13" t="str">
         <x:v>FE-CREATE-SUBJECT-02</x:v>
       </x:c>
       <x:c r="K99" s="13" t="str">
-        <x:v>待完成</x:v>
+        <x:v>已完成</x:v>
       </x:c>
       <x:c r="L99" s="13" t="str">
         <x:v>08-22～08-24</x:v>
       </x:c>
       <x:c r="M99" s="13" t="str">
-        <x:v>—</x:v>
+        <x:v>2026-08-21</x:v>
       </x:c>
       <x:c r="N99" s="13" t="str">
         <x:v>job/subject/variant/asset均为UUID；创建请求带idempotency_key；记录设置/Skill/模型版本</x:v>
@@ -6073,25 +6073,25 @@
         <x:v>前端</x:v>
       </x:c>
       <x:c r="G100" s="13" t="str">
-        <x:v>完成创建页主体编辑区中英文文案</x:v>
+        <x:v>完成批量输入中英文文案</x:v>
       </x:c>
       <x:c r="H100" s="13" t="str">
-        <x:v>en/zh词条</x:v>
+        <x:v>说明、示例、识别数量和错误词条</x:v>
       </x:c>
       <x:c r="I100" s="13" t="str">
-        <x:v>切换语言后字段含义、按钮和错误保持一致</x:v>
+        <x:v>切换语言后输入值和解析结果不变</x:v>
       </x:c>
       <x:c r="J100" s="13" t="str">
         <x:v>—</x:v>
       </x:c>
       <x:c r="K100" s="13" t="str">
-        <x:v>待完成</x:v>
+        <x:v>已完成</x:v>
       </x:c>
       <x:c r="L100" s="13" t="str">
         <x:v>08-22～08-24</x:v>
       </x:c>
       <x:c r="M100" s="13" t="str">
-        <x:v>—</x:v>
+        <x:v>2026-08-21</x:v>
       </x:c>
       <x:c r="N100" s="13" t="str">
         <x:v>job/subject/variant/asset均为UUID；创建请求带idempotency_key；记录设置/Skill/模型版本</x:v>
@@ -6241,25 +6241,25 @@
         <x:v>前端</x:v>
       </x:c>
       <x:c r="G103" s="13" t="str">
-        <x:v>建立主体颜色设置路由与页面边界</x:v>
+        <x:v>建立/create主体颜色设置区</x:v>
       </x:c>
       <x:c r="H103" s="13" t="str">
-        <x:v>主体颜色设置路由、页面组件和Metadata</x:v>
+        <x:v>同一创建页内的主体颜色区块</x:v>
       </x:c>
       <x:c r="I103" s="13" t="str">
-        <x:v>直接访问路由可渲染；未授权跳转符合PRD；无运行时错误</x:v>
+        <x:v>纯色与渐变均在/create内完成</x:v>
       </x:c>
       <x:c r="J103" s="13" t="str">
         <x:v>—</x:v>
       </x:c>
       <x:c r="K103" s="13" t="str">
-        <x:v>待完成</x:v>
+        <x:v>已完成</x:v>
       </x:c>
       <x:c r="L103" s="13" t="str">
         <x:v>08-23～08-25</x:v>
       </x:c>
       <x:c r="M103" s="13" t="str">
-        <x:v>—</x:v>
+        <x:v>2026-08-21</x:v>
       </x:c>
       <x:c r="N103" s="13" t="str">
         <x:v>job/subject/variant/asset均为UUID；创建请求带idempotency_key；记录设置/Skill/模型版本</x:v>
@@ -6309,13 +6309,13 @@
         <x:v>FE-CREATE-COLOR-01</x:v>
       </x:c>
       <x:c r="K104" s="13" t="str">
-        <x:v>待完成</x:v>
+        <x:v>已完成</x:v>
       </x:c>
       <x:c r="L104" s="13" t="str">
         <x:v>08-23～08-25</x:v>
       </x:c>
       <x:c r="M104" s="13" t="str">
-        <x:v>—</x:v>
+        <x:v>2026-08-21</x:v>
       </x:c>
       <x:c r="N104" s="13" t="str">
         <x:v>job/subject/variant/asset均为UUID；创建请求带idempotency_key；记录设置/Skill/模型版本</x:v>
@@ -6365,13 +6365,13 @@
         <x:v>—</x:v>
       </x:c>
       <x:c r="K105" s="13" t="str">
-        <x:v>待完成</x:v>
+        <x:v>已完成</x:v>
       </x:c>
       <x:c r="L105" s="13" t="str">
         <x:v>08-23～08-25</x:v>
       </x:c>
       <x:c r="M105" s="13" t="str">
-        <x:v>—</x:v>
+        <x:v>2026-08-21</x:v>
       </x:c>
       <x:c r="N105" s="13" t="str">
         <x:v>job/subject/variant/asset均为UUID；创建请求带idempotency_key；记录设置/Skill/模型版本</x:v>
@@ -6421,13 +6421,13 @@
         <x:v>—</x:v>
       </x:c>
       <x:c r="K106" s="13" t="str">
-        <x:v>待完成</x:v>
+        <x:v>已完成</x:v>
       </x:c>
       <x:c r="L106" s="13" t="str">
         <x:v>08-23～08-25</x:v>
       </x:c>
       <x:c r="M106" s="13" t="str">
-        <x:v>—</x:v>
+        <x:v>2026-08-21</x:v>
       </x:c>
       <x:c r="N106" s="13" t="str">
         <x:v>job/subject/variant/asset均为UUID；创建请求带idempotency_key；记录设置/Skill/模型版本</x:v>
@@ -6477,13 +6477,13 @@
         <x:v>—</x:v>
       </x:c>
       <x:c r="K107" s="13" t="str">
-        <x:v>待完成</x:v>
+        <x:v>已完成</x:v>
       </x:c>
       <x:c r="L107" s="13" t="str">
         <x:v>08-23～08-25</x:v>
       </x:c>
       <x:c r="M107" s="13" t="str">
-        <x:v>—</x:v>
+        <x:v>2026-08-21</x:v>
       </x:c>
       <x:c r="N107" s="13" t="str">
         <x:v>job/subject/variant/asset均为UUID；创建请求带idempotency_key；记录设置/Skill/模型版本</x:v>
@@ -6521,25 +6521,25 @@
         <x:v>前端</x:v>
       </x:c>
       <x:c r="G108" s="13" t="str">
-        <x:v>实现单主体颜色覆盖</x:v>
+        <x:v>实现全部颜色HEX手动输入</x:v>
       </x:c>
       <x:c r="H108" s="13" t="str">
-        <x:v>override开关和颜色值</x:v>
+        <x:v>主体与背景的纯色、渐变起始色、渐变结束色均提供#RRGGBB输入</x:v>
       </x:c>
       <x:c r="I108" s="13" t="str">
-        <x:v>关闭后回退全局颜色</x:v>
+        <x:v>每个颜色同时支持取色器和手输；字段有双语标签；无效格式提示且不提交</x:v>
       </x:c>
       <x:c r="J108" s="13" t="str">
         <x:v>—</x:v>
       </x:c>
       <x:c r="K108" s="13" t="str">
-        <x:v>待完成</x:v>
+        <x:v>已完成</x:v>
       </x:c>
       <x:c r="L108" s="13" t="str">
         <x:v>08-23～08-25</x:v>
       </x:c>
       <x:c r="M108" s="13" t="str">
-        <x:v>—</x:v>
+        <x:v>2026-08-21</x:v>
       </x:c>
       <x:c r="N108" s="13" t="str">
         <x:v>job/subject/variant/asset均为UUID；创建请求带idempotency_key；记录设置/Skill/模型版本</x:v>
@@ -6589,13 +6589,13 @@
         <x:v>FE-CREATE-COLOR-02</x:v>
       </x:c>
       <x:c r="K109" s="13" t="str">
-        <x:v>待完成</x:v>
+        <x:v>已完成</x:v>
       </x:c>
       <x:c r="L109" s="13" t="str">
         <x:v>08-23～08-25</x:v>
       </x:c>
       <x:c r="M109" s="13" t="str">
-        <x:v>—</x:v>
+        <x:v>2026-08-21</x:v>
       </x:c>
       <x:c r="N109" s="13" t="str">
         <x:v>job/subject/variant/asset均为UUID；创建请求带idempotency_key；记录设置/Skill/模型版本</x:v>
@@ -6701,13 +6701,13 @@
         <x:v>FE-CREATE-COLOR-02</x:v>
       </x:c>
       <x:c r="K111" s="13" t="str">
-        <x:v>待完成</x:v>
+        <x:v>已完成</x:v>
       </x:c>
       <x:c r="L111" s="13" t="str">
         <x:v>08-23～08-25</x:v>
       </x:c>
       <x:c r="M111" s="13" t="str">
-        <x:v>—</x:v>
+        <x:v>2026-08-21</x:v>
       </x:c>
       <x:c r="N111" s="13" t="str">
         <x:v>job/subject/variant/asset均为UUID；创建请求带idempotency_key；记录设置/Skill/模型版本</x:v>
@@ -6757,13 +6757,13 @@
         <x:v>—</x:v>
       </x:c>
       <x:c r="K112" s="13" t="str">
-        <x:v>待完成</x:v>
+        <x:v>已完成</x:v>
       </x:c>
       <x:c r="L112" s="13" t="str">
         <x:v>08-23～08-25</x:v>
       </x:c>
       <x:c r="M112" s="13" t="str">
-        <x:v>—</x:v>
+        <x:v>2026-08-21</x:v>
       </x:c>
       <x:c r="N112" s="13" t="str">
         <x:v>job/subject/variant/asset均为UUID；创建请求带idempotency_key；记录设置/Skill/模型版本</x:v>
@@ -6913,25 +6913,25 @@
         <x:v>前端</x:v>
       </x:c>
       <x:c r="G115" s="13" t="str">
-        <x:v>建立背景设置路由与页面边界</x:v>
+        <x:v>建立/create背景设置区</x:v>
       </x:c>
       <x:c r="H115" s="13" t="str">
-        <x:v>背景设置路由、页面组件和Metadata</x:v>
+        <x:v>同一创建页内的背景开关与条件区块</x:v>
       </x:c>
       <x:c r="I115" s="13" t="str">
-        <x:v>直接访问路由可渲染；未授权跳转符合PRD；无运行时错误</x:v>
+        <x:v>关闭背景时隐藏背景分类与颜色设置</x:v>
       </x:c>
       <x:c r="J115" s="13" t="str">
         <x:v>—</x:v>
       </x:c>
       <x:c r="K115" s="13" t="str">
-        <x:v>待完成</x:v>
+        <x:v>已完成</x:v>
       </x:c>
       <x:c r="L115" s="13" t="str">
         <x:v>08-23～08-25</x:v>
       </x:c>
       <x:c r="M115" s="13" t="str">
-        <x:v>—</x:v>
+        <x:v>2026-08-21</x:v>
       </x:c>
       <x:c r="N115" s="13" t="str">
         <x:v>job/subject/variant/asset均为UUID；创建请求带idempotency_key；记录设置/Skill/模型版本</x:v>
@@ -6981,13 +6981,13 @@
         <x:v>FE-CREATE-BG-01</x:v>
       </x:c>
       <x:c r="K116" s="13" t="str">
-        <x:v>待完成</x:v>
+        <x:v>已完成</x:v>
       </x:c>
       <x:c r="L116" s="13" t="str">
         <x:v>08-23～08-25</x:v>
       </x:c>
       <x:c r="M116" s="13" t="str">
-        <x:v>—</x:v>
+        <x:v>2026-08-21</x:v>
       </x:c>
       <x:c r="N116" s="13" t="str">
         <x:v>job/subject/variant/asset均为UUID；创建请求带idempotency_key；记录设置/Skill/模型版本</x:v>
@@ -7037,13 +7037,13 @@
         <x:v>—</x:v>
       </x:c>
       <x:c r="K117" s="13" t="str">
-        <x:v>待完成</x:v>
+        <x:v>已完成</x:v>
       </x:c>
       <x:c r="L117" s="13" t="str">
         <x:v>08-23～08-25</x:v>
       </x:c>
       <x:c r="M117" s="13" t="str">
-        <x:v>—</x:v>
+        <x:v>2026-08-21</x:v>
       </x:c>
       <x:c r="N117" s="13" t="str">
         <x:v>job/subject/variant/asset均为UUID；创建请求带idempotency_key；记录设置/Skill/模型版本</x:v>
@@ -7081,25 +7081,25 @@
         <x:v>前端</x:v>
       </x:c>
       <x:c r="G118" s="13" t="str">
-        <x:v>实现背景容器选择</x:v>
+        <x:v>实现图标背景形状三选一</x:v>
       </x:c>
       <x:c r="H118" s="13" t="str">
-        <x:v>circle/square/rounded-square/pill</x:v>
+        <x:v>图标背景区域、背景颜色之前显示 Rounded、Circular、Square</x:v>
       </x:c>
       <x:c r="I118" s="13" t="str">
-        <x:v>只能单选允许值</x:v>
+        <x:v>开启背景后仅显示三种且单选；顺序为Rounded→Circular→Square；无背景由开关控制；不显示胶囊形</x:v>
       </x:c>
       <x:c r="J118" s="13" t="str">
         <x:v>—</x:v>
       </x:c>
       <x:c r="K118" s="13" t="str">
-        <x:v>待完成</x:v>
+        <x:v>已完成</x:v>
       </x:c>
       <x:c r="L118" s="13" t="str">
         <x:v>08-23～08-25</x:v>
       </x:c>
       <x:c r="M118" s="13" t="str">
-        <x:v>—</x:v>
+        <x:v>2026-08-21</x:v>
       </x:c>
       <x:c r="N118" s="13" t="str">
         <x:v>job/subject/variant/asset均为UUID；创建请求带idempotency_key；记录设置/Skill/模型版本</x:v>
@@ -7137,25 +7137,25 @@
         <x:v>前端</x:v>
       </x:c>
       <x:c r="G119" s="13" t="str">
-        <x:v>实现背景纯色</x:v>
+        <x:v>实现背景纯色与手动输入</x:v>
       </x:c>
       <x:c r="H119" s="13" t="str">
-        <x:v>背景HEX输入</x:v>
+        <x:v>背景纯色提供取色器和#RRGGBB手动输入</x:v>
       </x:c>
       <x:c r="I119" s="13" t="str">
-        <x:v>与主体颜色字段分离</x:v>
+        <x:v>仅开启背景时展示和提交；无效HEX不得进入请求</x:v>
       </x:c>
       <x:c r="J119" s="13" t="str">
         <x:v>—</x:v>
       </x:c>
       <x:c r="K119" s="13" t="str">
-        <x:v>待完成</x:v>
+        <x:v>已完成</x:v>
       </x:c>
       <x:c r="L119" s="13" t="str">
         <x:v>08-23～08-25</x:v>
       </x:c>
       <x:c r="M119" s="13" t="str">
-        <x:v>—</x:v>
+        <x:v>2026-08-21</x:v>
       </x:c>
       <x:c r="N119" s="13" t="str">
         <x:v>job/subject/variant/asset均为UUID；创建请求带idempotency_key；记录设置/Skill/模型版本</x:v>
@@ -7193,25 +7193,25 @@
         <x:v>前端</x:v>
       </x:c>
       <x:c r="G120" s="13" t="str">
-        <x:v>实现背景渐变</x:v>
+        <x:v>实现背景渐变与手动输入</x:v>
       </x:c>
       <x:c r="H120" s="13" t="str">
-        <x:v>两色和方向</x:v>
+        <x:v>渐变起始色、结束色均提供取色器和#RRGGBB手动输入，并支持方向</x:v>
       </x:c>
       <x:c r="I120" s="13" t="str">
-        <x:v>仅背景开启时提交</x:v>
+        <x:v>两个颜色均可独立手输；仅背景开启且渐变模式时提交</x:v>
       </x:c>
       <x:c r="J120" s="13" t="str">
         <x:v>—</x:v>
       </x:c>
       <x:c r="K120" s="13" t="str">
-        <x:v>待完成</x:v>
+        <x:v>已完成</x:v>
       </x:c>
       <x:c r="L120" s="13" t="str">
         <x:v>08-23～08-25</x:v>
       </x:c>
       <x:c r="M120" s="13" t="str">
-        <x:v>—</x:v>
+        <x:v>2026-08-21</x:v>
       </x:c>
       <x:c r="N120" s="13" t="str">
         <x:v>job/subject/variant/asset均为UUID；创建请求带idempotency_key；记录设置/Skill/模型版本</x:v>
@@ -7261,13 +7261,13 @@
         <x:v>FE-CREATE-BG-02</x:v>
       </x:c>
       <x:c r="K121" s="13" t="str">
-        <x:v>待完成</x:v>
+        <x:v>已完成</x:v>
       </x:c>
       <x:c r="L121" s="13" t="str">
         <x:v>08-23～08-25</x:v>
       </x:c>
       <x:c r="M121" s="13" t="str">
-        <x:v>—</x:v>
+        <x:v>2026-08-21</x:v>
       </x:c>
       <x:c r="N121" s="13" t="str">
         <x:v>job/subject/variant/asset均为UUID；创建请求带idempotency_key；记录设置/Skill/模型版本</x:v>
@@ -7373,13 +7373,13 @@
         <x:v>FE-CREATE-BG-02</x:v>
       </x:c>
       <x:c r="K123" s="13" t="str">
-        <x:v>待完成</x:v>
+        <x:v>已完成</x:v>
       </x:c>
       <x:c r="L123" s="13" t="str">
         <x:v>08-23～08-25</x:v>
       </x:c>
       <x:c r="M123" s="13" t="str">
-        <x:v>—</x:v>
+        <x:v>2026-08-21</x:v>
       </x:c>
       <x:c r="N123" s="13" t="str">
         <x:v>job/subject/variant/asset均为UUID；创建请求带idempotency_key；记录设置/Skill/模型版本</x:v>
@@ -7429,13 +7429,13 @@
         <x:v>—</x:v>
       </x:c>
       <x:c r="K124" s="13" t="str">
-        <x:v>待完成</x:v>
+        <x:v>已完成</x:v>
       </x:c>
       <x:c r="L124" s="13" t="str">
         <x:v>08-23～08-25</x:v>
       </x:c>
       <x:c r="M124" s="13" t="str">
-        <x:v>—</x:v>
+        <x:v>2026-08-21</x:v>
       </x:c>
       <x:c r="N124" s="13" t="str">
         <x:v>job/subject/variant/asset均为UUID；创建请求带idempotency_key；记录设置/Skill/模型版本</x:v>
@@ -7576,7 +7576,7 @@
         <x:v>GEN-004</x:v>
       </x:c>
       <x:c r="D127" s="13" t="str">
-        <x:v>6组25项设置</x:v>
+        <x:v>图标设计风格</x:v>
       </x:c>
       <x:c r="E127" s="13" t="str">
         <x:v>FE-CREATE-SETTINGS-01</x:v>
@@ -7585,25 +7585,25 @@
         <x:v>前端</x:v>
       </x:c>
       <x:c r="G127" s="13" t="str">
-        <x:v>建立核心设置区路由与页面边界</x:v>
+        <x:v>重构创建页图标设计风格区</x:v>
       </x:c>
       <x:c r="H127" s="13" t="str">
-        <x:v>核心设置区路由、页面组件和Metadata</x:v>
+        <x:v>风格预设 + 风格微调的页面结构</x:v>
       </x:c>
       <x:c r="I127" s="13" t="str">
-        <x:v>直接访问路由可渲染；未授权跳转符合PRD；无运行时错误</x:v>
+        <x:v>不再展示6维/25项参数；背景、颜色、尺寸保持独立</x:v>
       </x:c>
       <x:c r="J127" s="13" t="str">
         <x:v>—</x:v>
       </x:c>
       <x:c r="K127" s="13" t="str">
-        <x:v>待完成</x:v>
+        <x:v>已完成</x:v>
       </x:c>
       <x:c r="L127" s="13" t="str">
         <x:v>08-24～08-26</x:v>
       </x:c>
       <x:c r="M127" s="13" t="str">
-        <x:v>—</x:v>
+        <x:v>2026-08-22</x:v>
       </x:c>
       <x:c r="N127" s="13" t="str">
         <x:v>job/subject/variant/asset均为UUID；创建请求带idempotency_key；记录设置/Skill/模型版本</x:v>
@@ -7632,7 +7632,7 @@
         <x:v>GEN-004</x:v>
       </x:c>
       <x:c r="D128" s="13" t="str">
-        <x:v>6组25项设置</x:v>
+        <x:v>图标设计风格</x:v>
       </x:c>
       <x:c r="E128" s="13" t="str">
         <x:v>FE-CREATE-SETTINGS-02</x:v>
@@ -7641,25 +7641,25 @@
         <x:v>前端</x:v>
       </x:c>
       <x:c r="G128" s="13" t="str">
-        <x:v>定义核心设置区页面状态模型</x:v>
+        <x:v>定义图标设计风格页面状态模型</x:v>
       </x:c>
       <x:c r="H128" s="13" t="str">
-        <x:v>页面状态类型与初始化逻辑</x:v>
+        <x:v>preset、strokeWeight、cornerStyle、detailLevel状态</x:v>
       </x:c>
       <x:c r="I128" s="13" t="str">
-        <x:v>每个状态只有一个含义；刷新后可恢复服务端状态</x:v>
+        <x:v>每个状态有唯一含义并能直接提交style</x:v>
       </x:c>
       <x:c r="J128" s="13" t="str">
         <x:v>FE-CREATE-SETTINGS-01</x:v>
       </x:c>
       <x:c r="K128" s="13" t="str">
-        <x:v>待完成</x:v>
+        <x:v>已完成</x:v>
       </x:c>
       <x:c r="L128" s="13" t="str">
         <x:v>08-24～08-26</x:v>
       </x:c>
       <x:c r="M128" s="13" t="str">
-        <x:v>—</x:v>
+        <x:v>2026-08-22</x:v>
       </x:c>
       <x:c r="N128" s="13" t="str">
         <x:v>job/subject/variant/asset均为UUID；创建请求带idempotency_key；记录设置/Skill/模型版本</x:v>
@@ -7688,7 +7688,7 @@
         <x:v>GEN-004</x:v>
       </x:c>
       <x:c r="D129" s="13" t="str">
-        <x:v>6组25项设置</x:v>
+        <x:v>图标设计风格</x:v>
       </x:c>
       <x:c r="E129" s="13" t="str">
         <x:v>FE-CREATE-SETTINGS-03</x:v>
@@ -7697,25 +7697,25 @@
         <x:v>前端</x:v>
       </x:c>
       <x:c r="G129" s="13" t="str">
-        <x:v>从服务端/共享配置渲染设置</x:v>
+        <x:v>从设置接口渲染5个风格预设</x:v>
       </x:c>
       <x:c r="H129" s="13" t="str">
-        <x:v>版本、6组、25项</x:v>
+        <x:v>极简线性、圆润线性、实心符号、双色分层、粗线几何</x:v>
       </x:c>
       <x:c r="I129" s="13" t="str">
-        <x:v>不在页面重复硬编码目录</x:v>
+        <x:v>预设名称、说明与顺序来自共享配置</x:v>
       </x:c>
       <x:c r="J129" s="13" t="str">
         <x:v>—</x:v>
       </x:c>
       <x:c r="K129" s="13" t="str">
-        <x:v>待完成</x:v>
+        <x:v>已完成</x:v>
       </x:c>
       <x:c r="L129" s="13" t="str">
         <x:v>08-24～08-26</x:v>
       </x:c>
       <x:c r="M129" s="13" t="str">
-        <x:v>—</x:v>
+        <x:v>2026-08-22</x:v>
       </x:c>
       <x:c r="N129" s="13" t="str">
         <x:v>job/subject/variant/asset均为UUID；创建请求带idempotency_key；记录设置/Skill/模型版本</x:v>
@@ -7744,7 +7744,7 @@
         <x:v>GEN-004</x:v>
       </x:c>
       <x:c r="D130" s="13" t="str">
-        <x:v>6组25项设置</x:v>
+        <x:v>图标设计风格</x:v>
       </x:c>
       <x:c r="E130" s="13" t="str">
         <x:v>FE-CREATE-SETTINGS-04</x:v>
@@ -7753,25 +7753,25 @@
         <x:v>前端</x:v>
       </x:c>
       <x:c r="G130" s="13" t="str">
-        <x:v>实现每组单选</x:v>
+        <x:v>渲染3组风格微调并支持单选</x:v>
       </x:c>
       <x:c r="H130" s="13" t="str">
-        <x:v>graphicStructure等6字段</x:v>
+        <x:v>线条粗细、转角语言、细节密度</x:v>
       </x:c>
       <x:c r="I130" s="13" t="str">
-        <x:v>每组始终恰好一个值</x:v>
+        <x:v>每组恰好一个选中值并写入style</x:v>
       </x:c>
       <x:c r="J130" s="13" t="str">
         <x:v>—</x:v>
       </x:c>
       <x:c r="K130" s="13" t="str">
-        <x:v>待完成</x:v>
+        <x:v>已完成</x:v>
       </x:c>
       <x:c r="L130" s="13" t="str">
         <x:v>08-24～08-26</x:v>
       </x:c>
       <x:c r="M130" s="13" t="str">
-        <x:v>—</x:v>
+        <x:v>2026-08-22</x:v>
       </x:c>
       <x:c r="N130" s="13" t="str">
         <x:v>job/subject/variant/asset均为UUID；创建请求带idempotency_key；记录设置/Skill/模型版本</x:v>
@@ -7800,7 +7800,7 @@
         <x:v>GEN-004</x:v>
       </x:c>
       <x:c r="D131" s="13" t="str">
-        <x:v>6组25项设置</x:v>
+        <x:v>图标设计风格</x:v>
       </x:c>
       <x:c r="E131" s="13" t="str">
         <x:v>FE-CREATE-SETTINGS-05</x:v>
@@ -7809,25 +7809,25 @@
         <x:v>前端</x:v>
       </x:c>
       <x:c r="G131" s="13" t="str">
-        <x:v>实现设置摘要</x:v>
+        <x:v>展示设计风格选择状态</x:v>
       </x:c>
       <x:c r="H131" s="13" t="str">
-        <x:v>人类可读双语摘要</x:v>
+        <x:v>选中勾选、aria-pressed与批次风格锁定提示</x:v>
       </x:c>
       <x:c r="I131" s="13" t="str">
-        <x:v>摘要值与提交值一致</x:v>
+        <x:v>视觉状态、无障碍状态和提交值一致</x:v>
       </x:c>
       <x:c r="J131" s="13" t="str">
         <x:v>—</x:v>
       </x:c>
       <x:c r="K131" s="13" t="str">
-        <x:v>待完成</x:v>
+        <x:v>已完成</x:v>
       </x:c>
       <x:c r="L131" s="13" t="str">
         <x:v>08-24～08-26</x:v>
       </x:c>
       <x:c r="M131" s="13" t="str">
-        <x:v>—</x:v>
+        <x:v>2026-08-22</x:v>
       </x:c>
       <x:c r="N131" s="13" t="str">
         <x:v>job/subject/variant/asset均为UUID；创建请求带idempotency_key；记录设置/Skill/模型版本</x:v>
@@ -7856,7 +7856,7 @@
         <x:v>GEN-004</x:v>
       </x:c>
       <x:c r="D132" s="13" t="str">
-        <x:v>6组25项设置</x:v>
+        <x:v>图标设计风格</x:v>
       </x:c>
       <x:c r="E132" s="13" t="str">
         <x:v>FE-CREATE-SETTINGS-06</x:v>
@@ -7865,25 +7865,25 @@
         <x:v>前端</x:v>
       </x:c>
       <x:c r="G132" s="13" t="str">
-        <x:v>处理设置版本过期</x:v>
+        <x:v>将背景设置与设计风格分离</x:v>
       </x:c>
       <x:c r="H132" s="13" t="str">
-        <x:v>刷新配置并保留可映射选择</x:v>
+        <x:v>背景形状仅在图标背景区设置</x:v>
       </x:c>
       <x:c r="I132" s="13" t="str">
-        <x:v>无法映射时明确要求重选</x:v>
+        <x:v>Rounded/Circular/Square不再被当作图标本体风格</x:v>
       </x:c>
       <x:c r="J132" s="13" t="str">
         <x:v>—</x:v>
       </x:c>
       <x:c r="K132" s="13" t="str">
-        <x:v>待完成</x:v>
+        <x:v>已完成</x:v>
       </x:c>
       <x:c r="L132" s="13" t="str">
         <x:v>08-24～08-26</x:v>
       </x:c>
       <x:c r="M132" s="13" t="str">
-        <x:v>—</x:v>
+        <x:v>2026-08-22</x:v>
       </x:c>
       <x:c r="N132" s="13" t="str">
         <x:v>job/subject/variant/asset均为UUID；创建请求带idempotency_key；记录设置/Skill/模型版本</x:v>
@@ -7912,7 +7912,7 @@
         <x:v>GEN-004</x:v>
       </x:c>
       <x:c r="D133" s="13" t="str">
-        <x:v>6组25项设置</x:v>
+        <x:v>图标设计风格</x:v>
       </x:c>
       <x:c r="E133" s="13" t="str">
         <x:v>FE-CREATE-SETTINGS-07</x:v>
@@ -7921,25 +7921,25 @@
         <x:v>前端</x:v>
       </x:c>
       <x:c r="G133" s="13" t="str">
-        <x:v>接入核心设置区服务端接口</x:v>
+        <x:v>接入图标设计风格设置接口</x:v>
       </x:c>
       <x:c r="H133" s="13" t="str">
         <x:v>GET /api/generation/settings客户端适配器</x:v>
       </x:c>
       <x:c r="I133" s="13" t="str">
-        <x:v>请求字段与共享Schema一致；不在组件内拼装不受控请求</x:v>
+        <x:v>请求字段与共享Schema一致；组件不拼装不受控请求</x:v>
       </x:c>
       <x:c r="J133" s="13" t="str">
         <x:v>FE-CREATE-SETTINGS-02</x:v>
       </x:c>
       <x:c r="K133" s="13" t="str">
-        <x:v>待完成</x:v>
+        <x:v>已完成</x:v>
       </x:c>
       <x:c r="L133" s="13" t="str">
         <x:v>08-24～08-26</x:v>
       </x:c>
       <x:c r="M133" s="13" t="str">
-        <x:v>—</x:v>
+        <x:v>2026-08-22</x:v>
       </x:c>
       <x:c r="N133" s="13" t="str">
         <x:v>job/subject/variant/asset均为UUID；创建请求带idempotency_key；记录设置/Skill/模型版本</x:v>
@@ -7968,7 +7968,7 @@
         <x:v>GEN-004</x:v>
       </x:c>
       <x:c r="D134" s="13" t="str">
-        <x:v>6组25项设置</x:v>
+        <x:v>图标设计风格</x:v>
       </x:c>
       <x:c r="E134" s="13" t="str">
         <x:v>FE-CREATE-SETTINGS-08</x:v>
@@ -7977,25 +7977,25 @@
         <x:v>前端</x:v>
       </x:c>
       <x:c r="G134" s="13" t="str">
-        <x:v>实现核心设置区加载状态</x:v>
+        <x:v>实现图标设计风格加载状态</x:v>
       </x:c>
       <x:c r="H134" s="13" t="str">
-        <x:v>骨架屏或进度反馈</x:v>
+        <x:v>设置接口加载反馈</x:v>
       </x:c>
       <x:c r="I134" s="13" t="str">
-        <x:v>请求期间有可感知反馈；重复操作被禁用</x:v>
+        <x:v>加载期间禁用生成提交</x:v>
       </x:c>
       <x:c r="J134" s="13" t="str">
         <x:v>FE-CREATE-SETTINGS-02</x:v>
       </x:c>
       <x:c r="K134" s="13" t="str">
-        <x:v>待完成</x:v>
+        <x:v>已完成</x:v>
       </x:c>
       <x:c r="L134" s="13" t="str">
         <x:v>08-24～08-26</x:v>
       </x:c>
       <x:c r="M134" s="13" t="str">
-        <x:v>—</x:v>
+        <x:v>2026-08-22</x:v>
       </x:c>
       <x:c r="N134" s="13" t="str">
         <x:v>job/subject/variant/asset均为UUID；创建请求带idempotency_key；记录设置/Skill/模型版本</x:v>
@@ -8024,7 +8024,7 @@
         <x:v>GEN-004</x:v>
       </x:c>
       <x:c r="D135" s="13" t="str">
-        <x:v>6组25项设置</x:v>
+        <x:v>图标设计风格</x:v>
       </x:c>
       <x:c r="E135" s="13" t="str">
         <x:v>FE-CREATE-SETTINGS-09</x:v>
@@ -8033,7 +8033,7 @@
         <x:v>前端</x:v>
       </x:c>
       <x:c r="G135" s="13" t="str">
-        <x:v>实现核心设置区错误映射</x:v>
+        <x:v>实现图标设计风格错误映射</x:v>
       </x:c>
       <x:c r="H135" s="13" t="str">
         <x:v>稳定错误码到双语用户文案的映射</x:v>
@@ -8045,13 +8045,13 @@
         <x:v>FE-CREATE-SETTINGS-02</x:v>
       </x:c>
       <x:c r="K135" s="13" t="str">
-        <x:v>待完成</x:v>
+        <x:v>已完成</x:v>
       </x:c>
       <x:c r="L135" s="13" t="str">
         <x:v>08-24～08-26</x:v>
       </x:c>
       <x:c r="M135" s="13" t="str">
-        <x:v>—</x:v>
+        <x:v>2026-08-22</x:v>
       </x:c>
       <x:c r="N135" s="13" t="str">
         <x:v>job/subject/variant/asset均为UUID；创建请求带idempotency_key；记录设置/Skill/模型版本</x:v>
@@ -8080,7 +8080,7 @@
         <x:v>GEN-004</x:v>
       </x:c>
       <x:c r="D136" s="13" t="str">
-        <x:v>6组25项设置</x:v>
+        <x:v>图标设计风格</x:v>
       </x:c>
       <x:c r="E136" s="13" t="str">
         <x:v>FE-CREATE-SETTINGS-10</x:v>
@@ -8089,25 +8089,25 @@
         <x:v>前端</x:v>
       </x:c>
       <x:c r="G136" s="13" t="str">
-        <x:v>完成核心设置区中英文文案</x:v>
+        <x:v>完成图标设计风格中英文文案</x:v>
       </x:c>
       <x:c r="H136" s="13" t="str">
-        <x:v>en/zh词条</x:v>
+        <x:v>预设、说明和微调项的en/zh词条</x:v>
       </x:c>
       <x:c r="I136" s="13" t="str">
-        <x:v>切换语言后字段含义、按钮和错误保持一致</x:v>
+        <x:v>切换语言后已选ID和表单状态不变</x:v>
       </x:c>
       <x:c r="J136" s="13" t="str">
         <x:v>—</x:v>
       </x:c>
       <x:c r="K136" s="13" t="str">
-        <x:v>待完成</x:v>
+        <x:v>已完成</x:v>
       </x:c>
       <x:c r="L136" s="13" t="str">
         <x:v>08-24～08-26</x:v>
       </x:c>
       <x:c r="M136" s="13" t="str">
-        <x:v>—</x:v>
+        <x:v>2026-08-22</x:v>
       </x:c>
       <x:c r="N136" s="13" t="str">
         <x:v>job/subject/variant/asset均为UUID；创建请求带idempotency_key；记录设置/Skill/模型版本</x:v>
@@ -8136,7 +8136,7 @@
         <x:v>GEN-004</x:v>
       </x:c>
       <x:c r="D137" s="13" t="str">
-        <x:v>6组25项设置</x:v>
+        <x:v>图标设计风格</x:v>
       </x:c>
       <x:c r="E137" s="13" t="str">
         <x:v>FE-CREATE-SETTINGS-11</x:v>
@@ -8145,13 +8145,13 @@
         <x:v>前端</x:v>
       </x:c>
       <x:c r="G137" s="13" t="str">
-        <x:v>完成核心设置区键盘与屏幕阅读器支持</x:v>
+        <x:v>完成图标设计风格键盘与屏幕阅读器支持</x:v>
       </x:c>
       <x:c r="H137" s="13" t="str">
-        <x:v>语义标签、焦点顺序、aria-live</x:v>
+        <x:v>语义标签、焦点顺序、aria-pressed</x:v>
       </x:c>
       <x:c r="I137" s="13" t="str">
-        <x:v>仅键盘可完成主流程；错误与状态可被读出</x:v>
+        <x:v>仅键盘可完成风格选择；选中状态可被读出</x:v>
       </x:c>
       <x:c r="J137" s="13" t="str">
         <x:v>—</x:v>
@@ -8192,7 +8192,7 @@
         <x:v>GEN-004</x:v>
       </x:c>
       <x:c r="D138" s="13" t="str">
-        <x:v>6组25项设置</x:v>
+        <x:v>图标设计风格</x:v>
       </x:c>
       <x:c r="E138" s="13" t="str">
         <x:v>FE-CREATE-SETTINGS-12</x:v>
@@ -8201,13 +8201,13 @@
         <x:v>前端</x:v>
       </x:c>
       <x:c r="G138" s="13" t="str">
-        <x:v>编写核心设置区组件测试</x:v>
+        <x:v>编写图标设计风格组件测试</x:v>
       </x:c>
       <x:c r="H138" s="13" t="str">
         <x:v>组件与交互测试</x:v>
       </x:c>
       <x:c r="I138" s="13" t="str">
-        <x:v>覆盖成功、校验失败、服务端失败和重复点击</x:v>
+        <x:v>覆盖预设、微调、双语切换和接口失败</x:v>
       </x:c>
       <x:c r="J138" s="13" t="str">
         <x:v>—</x:v>
@@ -8257,25 +8257,25 @@
         <x:v>前端</x:v>
       </x:c>
       <x:c r="G139" s="13" t="str">
-        <x:v>建立创建页提交区路由与页面边界</x:v>
+        <x:v>建立/create参考尺寸设置区</x:v>
       </x:c>
       <x:c r="H139" s="13" t="str">
-        <x:v>创建页提交区路由、页面组件和Metadata</x:v>
+        <x:v>同一创建页内的常用尺寸多选区块</x:v>
       </x:c>
       <x:c r="I139" s="13" t="str">
-        <x:v>直接访问路由可渲染；未授权跳转符合PRD；无运行时错误</x:v>
+        <x:v>只允许共享协议声明的固定尺寸</x:v>
       </x:c>
       <x:c r="J139" s="13" t="str">
         <x:v>—</x:v>
       </x:c>
       <x:c r="K139" s="13" t="str">
-        <x:v>待完成</x:v>
+        <x:v>已完成</x:v>
       </x:c>
       <x:c r="L139" s="13" t="str">
         <x:v>08-25～08-27</x:v>
       </x:c>
       <x:c r="M139" s="13" t="str">
-        <x:v>—</x:v>
+        <x:v>2026-08-21</x:v>
       </x:c>
       <x:c r="N139" s="13" t="str">
         <x:v>job/subject/variant/asset均为UUID；创建请求带idempotency_key；记录设置/Skill/模型版本</x:v>
@@ -8325,13 +8325,13 @@
         <x:v>FE-CREATE-SUBMIT-01</x:v>
       </x:c>
       <x:c r="K140" s="13" t="str">
-        <x:v>待完成</x:v>
+        <x:v>已完成</x:v>
       </x:c>
       <x:c r="L140" s="13" t="str">
         <x:v>08-25～08-27</x:v>
       </x:c>
       <x:c r="M140" s="13" t="str">
-        <x:v>—</x:v>
+        <x:v>2026-08-21</x:v>
       </x:c>
       <x:c r="N140" s="13" t="str">
         <x:v>job/subject/variant/asset均为UUID；创建请求带idempotency_key；记录设置/Skill/模型版本</x:v>
@@ -8369,25 +8369,25 @@
         <x:v>前端</x:v>
       </x:c>
       <x:c r="G141" s="13" t="str">
-        <x:v>实现常用尺寸多选</x:v>
+        <x:v>建立成功/失败/警告Toast组件</x:v>
       </x:c>
       <x:c r="H141" s="13" t="str">
-        <x:v>16至1024允许列表</x:v>
+        <x:v>提供success、error、warning三种语义样式；固定于底部水平居中；尺寸超限使用warning</x:v>
       </x:c>
       <x:c r="I141" s="13" t="str">
-        <x:v>至少选择1个；去重</x:v>
+        <x:v>三种类型具备独立颜色和图标；失败使用alert/assertive；成功和警告使用status/polite；默认6秒自动消失</x:v>
       </x:c>
       <x:c r="J141" s="13" t="str">
         <x:v>—</x:v>
       </x:c>
       <x:c r="K141" s="13" t="str">
-        <x:v>待完成</x:v>
+        <x:v>已完成</x:v>
       </x:c>
       <x:c r="L141" s="13" t="str">
         <x:v>08-25～08-27</x:v>
       </x:c>
       <x:c r="M141" s="13" t="str">
-        <x:v>—</x:v>
+        <x:v>2026-08-21</x:v>
       </x:c>
       <x:c r="N141" s="13" t="str">
         <x:v>job/subject/variant/asset均为UUID；创建请求带idempotency_key；记录设置/Skill/模型版本</x:v>
@@ -8425,25 +8425,25 @@
         <x:v>前端</x:v>
       </x:c>
       <x:c r="G142" s="13" t="str">
-        <x:v>显示预计点数</x:v>
+        <x:v>提交期间锁定表单</x:v>
       </x:c>
       <x:c r="H142" s="13" t="str">
-        <x:v>主体数×1点</x:v>
+        <x:v>防止重复点击生成按钮</x:v>
       </x:c>
       <x:c r="I142" s="13" t="str">
-        <x:v>随主体数实时更新</x:v>
+        <x:v>请求完成前不产生第二次提交</x:v>
       </x:c>
       <x:c r="J142" s="13" t="str">
         <x:v>—</x:v>
       </x:c>
       <x:c r="K142" s="13" t="str">
-        <x:v>待完成</x:v>
+        <x:v>已完成</x:v>
       </x:c>
       <x:c r="L142" s="13" t="str">
         <x:v>08-25～08-27</x:v>
       </x:c>
       <x:c r="M142" s="13" t="str">
-        <x:v>—</x:v>
+        <x:v>2026-08-21</x:v>
       </x:c>
       <x:c r="N142" s="13" t="str">
         <x:v>job/subject/variant/asset均为UUID；创建请求带idempotency_key；记录设置/Skill/模型版本</x:v>
@@ -8481,25 +8481,25 @@
         <x:v>前端</x:v>
       </x:c>
       <x:c r="G143" s="13" t="str">
-        <x:v>请求服务端报价</x:v>
+        <x:v>提交成功后进入结果页</x:v>
       </x:c>
       <x:c r="H143" s="13" t="str">
-        <x:v>服务端价格版本和余额</x:v>
+        <x:v>使用服务端返回jobId跳转</x:v>
       </x:c>
       <x:c r="I143" s="13" t="str">
-        <x:v>前端估算不作为扣点依据</x:v>
+        <x:v>不展示或请求点数报价</x:v>
       </x:c>
       <x:c r="J143" s="13" t="str">
         <x:v>—</x:v>
       </x:c>
       <x:c r="K143" s="13" t="str">
-        <x:v>待完成</x:v>
+        <x:v>已完成</x:v>
       </x:c>
       <x:c r="L143" s="13" t="str">
         <x:v>08-25～08-27</x:v>
       </x:c>
       <x:c r="M143" s="13" t="str">
-        <x:v>—</x:v>
+        <x:v>2026-08-21</x:v>
       </x:c>
       <x:c r="N143" s="13" t="str">
         <x:v>job/subject/variant/asset均为UUID；创建请求带idempotency_key；记录设置/Skill/模型版本</x:v>
@@ -8549,13 +8549,13 @@
         <x:v>—</x:v>
       </x:c>
       <x:c r="K144" s="13" t="str">
-        <x:v>待完成</x:v>
+        <x:v>已完成</x:v>
       </x:c>
       <x:c r="L144" s="13" t="str">
         <x:v>08-25～08-27</x:v>
       </x:c>
       <x:c r="M144" s="13" t="str">
-        <x:v>—</x:v>
+        <x:v>2026-08-21</x:v>
       </x:c>
       <x:c r="N144" s="13" t="str">
         <x:v>job/subject/variant/asset均为UUID；创建请求带idempotency_key；记录设置/Skill/模型版本</x:v>
@@ -8593,25 +8593,25 @@
         <x:v>前端</x:v>
       </x:c>
       <x:c r="G145" s="13" t="str">
-        <x:v>提交期间锁定表单</x:v>
+        <x:v>将尺寸写入生成请求</x:v>
       </x:c>
       <x:c r="H145" s="13" t="str">
-        <x:v>防重复提交</x:v>
+        <x:v>去重后的sizes数组</x:v>
       </x:c>
       <x:c r="I145" s="13" t="str">
-        <x:v>成功前不产生第二任务</x:v>
+        <x:v>请求中至少一个尺寸且只含固定允许值</x:v>
       </x:c>
       <x:c r="J145" s="13" t="str">
         <x:v>—</x:v>
       </x:c>
       <x:c r="K145" s="13" t="str">
-        <x:v>待完成</x:v>
+        <x:v>已完成</x:v>
       </x:c>
       <x:c r="L145" s="13" t="str">
         <x:v>08-25～08-27</x:v>
       </x:c>
       <x:c r="M145" s="13" t="str">
-        <x:v>—</x:v>
+        <x:v>2026-08-21</x:v>
       </x:c>
       <x:c r="N145" s="13" t="str">
         <x:v>job/subject/variant/asset均为UUID；创建请求带idempotency_key；记录设置/Skill/模型版本</x:v>
@@ -8649,25 +8649,25 @@
         <x:v>前端</x:v>
       </x:c>
       <x:c r="G146" s="13" t="str">
-        <x:v>处理余额不足</x:v>
+        <x:v>组装完整生成请求</x:v>
       </x:c>
       <x:c r="H146" s="13" t="str">
-        <x:v>展示所需/现有点数和购买入口</x:v>
+        <x:v>主体、颜色、背景、6组设置、尺寸和幂等键</x:v>
       </x:c>
       <x:c r="I146" s="13" t="str">
-        <x:v>草稿不丢失</x:v>
+        <x:v>请求不包含点数、报价或余额字段</x:v>
       </x:c>
       <x:c r="J146" s="13" t="str">
         <x:v>—</x:v>
       </x:c>
       <x:c r="K146" s="13" t="str">
-        <x:v>待完成</x:v>
+        <x:v>已完成</x:v>
       </x:c>
       <x:c r="L146" s="13" t="str">
         <x:v>08-25～08-27</x:v>
       </x:c>
       <x:c r="M146" s="13" t="str">
-        <x:v>—</x:v>
+        <x:v>2026-08-21</x:v>
       </x:c>
       <x:c r="N146" s="13" t="str">
         <x:v>job/subject/variant/asset均为UUID；创建请求带idempotency_key；记录设置/Skill/模型版本</x:v>
@@ -8708,22 +8708,22 @@
         <x:v>处理活动任务限制</x:v>
       </x:c>
       <x:c r="H147" s="13" t="str">
-        <x:v>引导现有任务详情</x:v>
+        <x:v>活动任务错误和已有任务提示</x:v>
       </x:c>
       <x:c r="I147" s="13" t="str">
-        <x:v>不重复扣点</x:v>
+        <x:v>不创建重复生成任务</x:v>
       </x:c>
       <x:c r="J147" s="13" t="str">
         <x:v>—</x:v>
       </x:c>
       <x:c r="K147" s="13" t="str">
-        <x:v>待完成</x:v>
+        <x:v>已完成</x:v>
       </x:c>
       <x:c r="L147" s="13" t="str">
         <x:v>08-25～08-27</x:v>
       </x:c>
       <x:c r="M147" s="13" t="str">
-        <x:v>—</x:v>
+        <x:v>2026-08-21</x:v>
       </x:c>
       <x:c r="N147" s="13" t="str">
         <x:v>job/subject/variant/asset均为UUID；创建请求带idempotency_key；记录设置/Skill/模型版本</x:v>
@@ -8764,22 +8764,22 @@
         <x:v>接入创建页提交区服务端接口</x:v>
       </x:c>
       <x:c r="H148" s="13" t="str">
-        <x:v>quote+POST /api/generation/jobs客户端适配器</x:v>
+        <x:v>POST /api/generation/jobs客户端适配器</x:v>
       </x:c>
       <x:c r="I148" s="13" t="str">
-        <x:v>请求字段与共享Schema一致；不在组件内拼装不受控请求</x:v>
+        <x:v>请求字段与共享Schema一致；不传点数字段</x:v>
       </x:c>
       <x:c r="J148" s="13" t="str">
         <x:v>FE-CREATE-SUBMIT-02</x:v>
       </x:c>
       <x:c r="K148" s="13" t="str">
-        <x:v>待完成</x:v>
+        <x:v>已完成</x:v>
       </x:c>
       <x:c r="L148" s="13" t="str">
         <x:v>08-25～08-27</x:v>
       </x:c>
       <x:c r="M148" s="13" t="str">
-        <x:v>—</x:v>
+        <x:v>2026-08-21</x:v>
       </x:c>
       <x:c r="N148" s="13" t="str">
         <x:v>job/subject/variant/asset均为UUID；创建请求带idempotency_key；记录设置/Skill/模型版本</x:v>
@@ -8817,25 +8817,25 @@
         <x:v>前端</x:v>
       </x:c>
       <x:c r="G149" s="13" t="str">
-        <x:v>实现创建页提交区加载状态</x:v>
+        <x:v>处理任务创建失败</x:v>
       </x:c>
       <x:c r="H149" s="13" t="str">
-        <x:v>骨架屏或进度反馈</x:v>
+        <x:v>稳定错误提示并解除提交锁定</x:v>
       </x:c>
       <x:c r="I149" s="13" t="str">
-        <x:v>请求期间有可感知反馈；重复操作被禁用</x:v>
+        <x:v>失败后保留全部设计输入且可再次提交</x:v>
       </x:c>
       <x:c r="J149" s="13" t="str">
         <x:v>FE-CREATE-SUBMIT-02</x:v>
       </x:c>
       <x:c r="K149" s="13" t="str">
-        <x:v>待完成</x:v>
+        <x:v>已完成</x:v>
       </x:c>
       <x:c r="L149" s="13" t="str">
         <x:v>08-25～08-27</x:v>
       </x:c>
       <x:c r="M149" s="13" t="str">
-        <x:v>—</x:v>
+        <x:v>2026-08-21</x:v>
       </x:c>
       <x:c r="N149" s="13" t="str">
         <x:v>job/subject/variant/asset均为UUID；创建请求带idempotency_key；记录设置/Skill/模型版本</x:v>
@@ -8885,13 +8885,13 @@
         <x:v>FE-CREATE-SUBMIT-02</x:v>
       </x:c>
       <x:c r="K150" s="13" t="str">
-        <x:v>待完成</x:v>
+        <x:v>已完成</x:v>
       </x:c>
       <x:c r="L150" s="13" t="str">
         <x:v>08-25～08-27</x:v>
       </x:c>
       <x:c r="M150" s="13" t="str">
-        <x:v>—</x:v>
+        <x:v>2026-08-21</x:v>
       </x:c>
       <x:c r="N150" s="13" t="str">
         <x:v>job/subject/variant/asset均为UUID；创建请求带idempotency_key；记录设置/Skill/模型版本</x:v>
@@ -8941,13 +8941,13 @@
         <x:v>—</x:v>
       </x:c>
       <x:c r="K151" s="13" t="str">
-        <x:v>待完成</x:v>
+        <x:v>已完成</x:v>
       </x:c>
       <x:c r="L151" s="13" t="str">
         <x:v>08-25～08-27</x:v>
       </x:c>
       <x:c r="M151" s="13" t="str">
-        <x:v>—</x:v>
+        <x:v>2026-08-21</x:v>
       </x:c>
       <x:c r="N151" s="13" t="str">
         <x:v>job/subject/variant/asset均为UUID；创建请求带idempotency_key；记录设置/Skill/模型版本</x:v>
@@ -8997,13 +8997,13 @@
         <x:v>—</x:v>
       </x:c>
       <x:c r="K152" s="13" t="str">
-        <x:v>待完成</x:v>
+        <x:v>已完成</x:v>
       </x:c>
       <x:c r="L152" s="13" t="str">
         <x:v>08-25～08-27</x:v>
       </x:c>
       <x:c r="M152" s="13" t="str">
-        <x:v>—</x:v>
+        <x:v>2026-08-21</x:v>
       </x:c>
       <x:c r="N152" s="13" t="str">
         <x:v>job/subject/variant/asset均为UUID；创建请求带idempotency_key；记录设置/Skill/模型版本</x:v>
@@ -9097,25 +9097,25 @@
         <x:v>前端</x:v>
       </x:c>
       <x:c r="G154" s="13" t="str">
-        <x:v>建立生成进度区路由与页面边界</x:v>
+        <x:v>建立结果页生成进度区</x:v>
       </x:c>
       <x:c r="H154" s="13" t="str">
-        <x:v>生成进度区路由、页面组件和Metadata</x:v>
+        <x:v>任务详情页内的进度条、百分比和提示文本</x:v>
       </x:c>
       <x:c r="I154" s="13" t="str">
-        <x:v>直接访问路由可渲染；未授权跳转符合PRD；无运行时错误</x:v>
+        <x:v>提交后进入结果页并持续展示真实服务端进度</x:v>
       </x:c>
       <x:c r="J154" s="13" t="str">
         <x:v>—</x:v>
       </x:c>
       <x:c r="K154" s="13" t="str">
-        <x:v>待完成</x:v>
+        <x:v>已完成</x:v>
       </x:c>
       <x:c r="L154" s="13" t="str">
         <x:v>08-26～08-28</x:v>
       </x:c>
       <x:c r="M154" s="13" t="str">
-        <x:v>—</x:v>
+        <x:v>2026-08-21</x:v>
       </x:c>
       <x:c r="N154" s="13" t="str">
         <x:v>job/subject/variant/asset均为UUID；创建请求带idempotency_key；记录设置/Skill/模型版本</x:v>
@@ -9165,13 +9165,13 @@
         <x:v>FE-PROGRESS-01</x:v>
       </x:c>
       <x:c r="K155" s="13" t="str">
-        <x:v>待完成</x:v>
+        <x:v>已完成</x:v>
       </x:c>
       <x:c r="L155" s="13" t="str">
         <x:v>08-26～08-28</x:v>
       </x:c>
       <x:c r="M155" s="13" t="str">
-        <x:v>—</x:v>
+        <x:v>2026-08-21</x:v>
       </x:c>
       <x:c r="N155" s="13" t="str">
         <x:v>job/subject/variant/asset均为UUID；创建请求带idempotency_key；记录设置/Skill/模型版本</x:v>
@@ -9221,13 +9221,13 @@
         <x:v>—</x:v>
       </x:c>
       <x:c r="K156" s="13" t="str">
-        <x:v>待完成</x:v>
+        <x:v>已完成</x:v>
       </x:c>
       <x:c r="L156" s="13" t="str">
         <x:v>08-26～08-28</x:v>
       </x:c>
       <x:c r="M156" s="13" t="str">
-        <x:v>—</x:v>
+        <x:v>2026-08-21</x:v>
       </x:c>
       <x:c r="N156" s="13" t="str">
         <x:v>job/subject/variant/asset均为UUID；创建请求带idempotency_key；记录设置/Skill/模型版本</x:v>
@@ -9277,13 +9277,13 @@
         <x:v>—</x:v>
       </x:c>
       <x:c r="K157" s="13" t="str">
-        <x:v>待完成</x:v>
+        <x:v>已完成</x:v>
       </x:c>
       <x:c r="L157" s="13" t="str">
         <x:v>08-26～08-28</x:v>
       </x:c>
       <x:c r="M157" s="13" t="str">
-        <x:v>—</x:v>
+        <x:v>2026-08-21</x:v>
       </x:c>
       <x:c r="N157" s="13" t="str">
         <x:v>job/subject/variant/asset均为UUID；创建请求带idempotency_key；记录设置/Skill/模型版本</x:v>
@@ -9333,13 +9333,13 @@
         <x:v>—</x:v>
       </x:c>
       <x:c r="K158" s="13" t="str">
-        <x:v>待完成</x:v>
+        <x:v>已完成</x:v>
       </x:c>
       <x:c r="L158" s="13" t="str">
         <x:v>08-26～08-28</x:v>
       </x:c>
       <x:c r="M158" s="13" t="str">
-        <x:v>—</x:v>
+        <x:v>2026-08-21</x:v>
       </x:c>
       <x:c r="N158" s="13" t="str">
         <x:v>job/subject/variant/asset均为UUID；创建请求带idempotency_key；记录设置/Skill/模型版本</x:v>
@@ -9389,13 +9389,13 @@
         <x:v>—</x:v>
       </x:c>
       <x:c r="K159" s="13" t="str">
-        <x:v>待完成</x:v>
+        <x:v>已完成</x:v>
       </x:c>
       <x:c r="L159" s="13" t="str">
         <x:v>08-26～08-28</x:v>
       </x:c>
       <x:c r="M159" s="13" t="str">
-        <x:v>—</x:v>
+        <x:v>2026-08-21</x:v>
       </x:c>
       <x:c r="N159" s="13" t="str">
         <x:v>job/subject/variant/asset均为UUID；创建请求带idempotency_key；记录设置/Skill/模型版本</x:v>
@@ -9445,13 +9445,13 @@
         <x:v>FE-PROGRESS-02</x:v>
       </x:c>
       <x:c r="K160" s="13" t="str">
-        <x:v>待完成</x:v>
+        <x:v>已完成</x:v>
       </x:c>
       <x:c r="L160" s="13" t="str">
         <x:v>08-26～08-28</x:v>
       </x:c>
       <x:c r="M160" s="13" t="str">
-        <x:v>—</x:v>
+        <x:v>2026-08-21</x:v>
       </x:c>
       <x:c r="N160" s="13" t="str">
         <x:v>job/subject/variant/asset均为UUID；创建请求带idempotency_key；记录设置/Skill/模型版本</x:v>
@@ -9501,13 +9501,13 @@
         <x:v>FE-PROGRESS-02</x:v>
       </x:c>
       <x:c r="K161" s="13" t="str">
-        <x:v>待完成</x:v>
+        <x:v>已完成</x:v>
       </x:c>
       <x:c r="L161" s="13" t="str">
         <x:v>08-26～08-28</x:v>
       </x:c>
       <x:c r="M161" s="13" t="str">
-        <x:v>—</x:v>
+        <x:v>2026-08-21</x:v>
       </x:c>
       <x:c r="N161" s="13" t="str">
         <x:v>job/subject/variant/asset均为UUID；创建请求带idempotency_key；记录设置/Skill/模型版本</x:v>
@@ -9557,13 +9557,13 @@
         <x:v>FE-PROGRESS-02</x:v>
       </x:c>
       <x:c r="K162" s="13" t="str">
-        <x:v>待完成</x:v>
+        <x:v>已完成</x:v>
       </x:c>
       <x:c r="L162" s="13" t="str">
         <x:v>08-26～08-28</x:v>
       </x:c>
       <x:c r="M162" s="13" t="str">
-        <x:v>—</x:v>
+        <x:v>2026-08-21</x:v>
       </x:c>
       <x:c r="N162" s="13" t="str">
         <x:v>job/subject/variant/asset均为UUID；创建请求带idempotency_key；记录设置/Skill/模型版本</x:v>
@@ -9613,13 +9613,13 @@
         <x:v>—</x:v>
       </x:c>
       <x:c r="K163" s="13" t="str">
-        <x:v>待完成</x:v>
+        <x:v>已完成</x:v>
       </x:c>
       <x:c r="L163" s="13" t="str">
         <x:v>08-26～08-28</x:v>
       </x:c>
       <x:c r="M163" s="13" t="str">
-        <x:v>—</x:v>
+        <x:v>2026-08-21</x:v>
       </x:c>
       <x:c r="N163" s="13" t="str">
         <x:v>job/subject/variant/asset均为UUID；创建请求带idempotency_key；记录设置/Skill/模型版本</x:v>
@@ -9781,13 +9781,13 @@
         <x:v>—</x:v>
       </x:c>
       <x:c r="K166" s="13" t="str">
-        <x:v>待完成</x:v>
+        <x:v>已完成</x:v>
       </x:c>
       <x:c r="L166" s="13" t="str">
         <x:v>09-03～09-06</x:v>
       </x:c>
       <x:c r="M166" s="13" t="str">
-        <x:v>—</x:v>
+        <x:v>2026-08-21</x:v>
       </x:c>
       <x:c r="N166" s="13" t="str">
         <x:v>job/subject/variant/asset均为UUID；创建请求带idempotency_key；记录设置/Skill/模型版本</x:v>
@@ -9837,13 +9837,13 @@
         <x:v>FE-RESULTS-01</x:v>
       </x:c>
       <x:c r="K167" s="13" t="str">
-        <x:v>待完成</x:v>
+        <x:v>已完成</x:v>
       </x:c>
       <x:c r="L167" s="13" t="str">
         <x:v>09-03～09-06</x:v>
       </x:c>
       <x:c r="M167" s="13" t="str">
-        <x:v>—</x:v>
+        <x:v>2026-08-21</x:v>
       </x:c>
       <x:c r="N167" s="13" t="str">
         <x:v>job/subject/variant/asset均为UUID；创建请求带idempotency_key；记录设置/Skill/模型版本</x:v>
@@ -9893,13 +9893,13 @@
         <x:v>—</x:v>
       </x:c>
       <x:c r="K168" s="13" t="str">
-        <x:v>待完成</x:v>
+        <x:v>已完成</x:v>
       </x:c>
       <x:c r="L168" s="13" t="str">
         <x:v>09-03～09-06</x:v>
       </x:c>
       <x:c r="M168" s="13" t="str">
-        <x:v>—</x:v>
+        <x:v>2026-08-21</x:v>
       </x:c>
       <x:c r="N168" s="13" t="str">
         <x:v>job/subject/variant/asset均为UUID；创建请求带idempotency_key；记录设置/Skill/模型版本</x:v>
@@ -9949,13 +9949,13 @@
         <x:v>—</x:v>
       </x:c>
       <x:c r="K169" s="13" t="str">
-        <x:v>待完成</x:v>
+        <x:v>已完成</x:v>
       </x:c>
       <x:c r="L169" s="13" t="str">
         <x:v>09-03～09-06</x:v>
       </x:c>
       <x:c r="M169" s="13" t="str">
-        <x:v>—</x:v>
+        <x:v>2026-08-21</x:v>
       </x:c>
       <x:c r="N169" s="13" t="str">
         <x:v>job/subject/variant/asset均为UUID；创建请求带idempotency_key；记录设置/Skill/模型版本</x:v>
@@ -10061,13 +10061,13 @@
         <x:v>—</x:v>
       </x:c>
       <x:c r="K171" s="13" t="str">
-        <x:v>待完成</x:v>
+        <x:v>已完成</x:v>
       </x:c>
       <x:c r="L171" s="13" t="str">
         <x:v>09-03～09-06</x:v>
       </x:c>
       <x:c r="M171" s="13" t="str">
-        <x:v>—</x:v>
+        <x:v>2026-08-21</x:v>
       </x:c>
       <x:c r="N171" s="13" t="str">
         <x:v>job/subject/variant/asset均为UUID；创建请求带idempotency_key；记录设置/Skill/模型版本</x:v>
@@ -10105,25 +10105,25 @@
         <x:v>前端</x:v>
       </x:c>
       <x:c r="G172" s="13" t="str">
-        <x:v>显示partial与退款提示</x:v>
+        <x:v>展示部分成功与失败状态</x:v>
       </x:c>
       <x:c r="H172" s="13" t="str">
-        <x:v>主体级失败和返还状态</x:v>
+        <x:v>主体级失败、缺失方案和可用结果状态</x:v>
       </x:c>
       <x:c r="I172" s="13" t="str">
-        <x:v>金额与creditSummary一致</x:v>
+        <x:v>不展示或计算点数、扣点与退款信息</x:v>
       </x:c>
       <x:c r="J172" s="13" t="str">
         <x:v>—</x:v>
       </x:c>
       <x:c r="K172" s="13" t="str">
-        <x:v>待完成</x:v>
+        <x:v>已完成</x:v>
       </x:c>
       <x:c r="L172" s="13" t="str">
         <x:v>09-03～09-06</x:v>
       </x:c>
       <x:c r="M172" s="13" t="str">
-        <x:v>—</x:v>
+        <x:v>2026-08-21</x:v>
       </x:c>
       <x:c r="N172" s="13" t="str">
         <x:v>job/subject/variant/asset均为UUID；创建请求带idempotency_key；记录设置/Skill/模型版本</x:v>
@@ -10173,13 +10173,13 @@
         <x:v>FE-RESULTS-02</x:v>
       </x:c>
       <x:c r="K173" s="13" t="str">
-        <x:v>待完成</x:v>
+        <x:v>已完成</x:v>
       </x:c>
       <x:c r="L173" s="13" t="str">
         <x:v>09-03～09-06</x:v>
       </x:c>
       <x:c r="M173" s="13" t="str">
-        <x:v>—</x:v>
+        <x:v>2026-08-21</x:v>
       </x:c>
       <x:c r="N173" s="13" t="str">
         <x:v>job/subject/variant/asset均为UUID；创建请求带idempotency_key；记录设置/Skill/模型版本</x:v>
@@ -10229,13 +10229,13 @@
         <x:v>FE-RESULTS-02</x:v>
       </x:c>
       <x:c r="K174" s="13" t="str">
-        <x:v>待完成</x:v>
+        <x:v>已完成</x:v>
       </x:c>
       <x:c r="L174" s="13" t="str">
         <x:v>09-03～09-06</x:v>
       </x:c>
       <x:c r="M174" s="13" t="str">
-        <x:v>—</x:v>
+        <x:v>2026-08-21</x:v>
       </x:c>
       <x:c r="N174" s="13" t="str">
         <x:v>job/subject/variant/asset均为UUID；创建请求带idempotency_key；记录设置/Skill/模型版本</x:v>
@@ -10285,13 +10285,13 @@
         <x:v>FE-RESULTS-02</x:v>
       </x:c>
       <x:c r="K175" s="13" t="str">
-        <x:v>待完成</x:v>
+        <x:v>已完成</x:v>
       </x:c>
       <x:c r="L175" s="13" t="str">
         <x:v>09-03～09-06</x:v>
       </x:c>
       <x:c r="M175" s="13" t="str">
-        <x:v>—</x:v>
+        <x:v>2026-08-21</x:v>
       </x:c>
       <x:c r="N175" s="13" t="str">
         <x:v>job/subject/variant/asset均为UUID；创建请求带idempotency_key；记录设置/Skill/模型版本</x:v>
@@ -10347,7 +10347,7 @@
         <x:v>09-03～09-06</x:v>
       </x:c>
       <x:c r="M176" s="13" t="str">
-        <x:v>2026-08-20</x:v>
+        <x:v>2026-08-21</x:v>
       </x:c>
       <x:c r="N176" s="13" t="str">
         <x:v>job/subject/variant/asset均为UUID；创建请求带idempotency_key；记录设置/Skill/模型版本</x:v>
@@ -11461,13 +11461,13 @@
         <x:v>—</x:v>
       </x:c>
       <x:c r="K196" s="13" t="str">
-        <x:v>待完成</x:v>
+        <x:v>已完成</x:v>
       </x:c>
       <x:c r="L196" s="13" t="str">
         <x:v>09-06～09-08</x:v>
       </x:c>
       <x:c r="M196" s="13" t="str">
-        <x:v>—</x:v>
+        <x:v>2026-08-21</x:v>
       </x:c>
       <x:c r="N196" s="13" t="str">
         <x:v>job/variant/asset UUID；archive_id UUID；归档键=用户+选择集+尺寸</x:v>
@@ -11909,13 +11909,13 @@
         <x:v>—</x:v>
       </x:c>
       <x:c r="K204" s="13" t="str">
-        <x:v>待完成</x:v>
+        <x:v>已完成</x:v>
       </x:c>
       <x:c r="L204" s="13" t="str">
         <x:v>09-08～09-10</x:v>
       </x:c>
       <x:c r="M204" s="13" t="str">
-        <x:v>—</x:v>
+        <x:v>2026-08-21</x:v>
       </x:c>
       <x:c r="N204" s="13" t="str">
         <x:v>job/variant/asset UUID；archive_id UUID；归档键=用户+选择集+尺寸</x:v>
@@ -11965,13 +11965,13 @@
         <x:v>FE-ZIP-01</x:v>
       </x:c>
       <x:c r="K205" s="13" t="str">
-        <x:v>待完成</x:v>
+        <x:v>已完成</x:v>
       </x:c>
       <x:c r="L205" s="13" t="str">
         <x:v>09-08～09-10</x:v>
       </x:c>
       <x:c r="M205" s="13" t="str">
-        <x:v>—</x:v>
+        <x:v>2026-08-21</x:v>
       </x:c>
       <x:c r="N205" s="13" t="str">
         <x:v>job/variant/asset UUID；archive_id UUID；归档键=用户+选择集+尺寸</x:v>
@@ -12021,13 +12021,13 @@
         <x:v>—</x:v>
       </x:c>
       <x:c r="K206" s="13" t="str">
-        <x:v>待完成</x:v>
+        <x:v>已完成</x:v>
       </x:c>
       <x:c r="L206" s="13" t="str">
         <x:v>09-08～09-10</x:v>
       </x:c>
       <x:c r="M206" s="13" t="str">
-        <x:v>—</x:v>
+        <x:v>2026-08-21</x:v>
       </x:c>
       <x:c r="N206" s="13" t="str">
         <x:v>job/variant/asset UUID；archive_id UUID；归档键=用户+选择集+尺寸</x:v>
@@ -12077,13 +12077,13 @@
         <x:v>—</x:v>
       </x:c>
       <x:c r="K207" s="13" t="str">
-        <x:v>待完成</x:v>
+        <x:v>已完成</x:v>
       </x:c>
       <x:c r="L207" s="13" t="str">
         <x:v>09-08～09-10</x:v>
       </x:c>
       <x:c r="M207" s="13" t="str">
-        <x:v>—</x:v>
+        <x:v>2026-08-21</x:v>
       </x:c>
       <x:c r="N207" s="13" t="str">
         <x:v>job/variant/asset UUID；archive_id UUID；归档键=用户+选择集+尺寸</x:v>
@@ -12133,13 +12133,13 @@
         <x:v>—</x:v>
       </x:c>
       <x:c r="K208" s="13" t="str">
-        <x:v>待完成</x:v>
+        <x:v>已完成</x:v>
       </x:c>
       <x:c r="L208" s="13" t="str">
         <x:v>09-08～09-10</x:v>
       </x:c>
       <x:c r="M208" s="13" t="str">
-        <x:v>—</x:v>
+        <x:v>2026-08-21</x:v>
       </x:c>
       <x:c r="N208" s="13" t="str">
         <x:v>job/variant/asset UUID；archive_id UUID；归档键=用户+选择集+尺寸</x:v>
@@ -12301,13 +12301,13 @@
         <x:v>—</x:v>
       </x:c>
       <x:c r="K211" s="13" t="str">
-        <x:v>待完成</x:v>
+        <x:v>已完成</x:v>
       </x:c>
       <x:c r="L211" s="13" t="str">
         <x:v>09-08～09-10</x:v>
       </x:c>
       <x:c r="M211" s="13" t="str">
-        <x:v>—</x:v>
+        <x:v>2026-08-21</x:v>
       </x:c>
       <x:c r="N211" s="13" t="str">
         <x:v>job/variant/asset UUID；archive_id UUID；归档键=用户+选择集+尺寸</x:v>
@@ -12357,13 +12357,13 @@
         <x:v>FE-ZIP-02</x:v>
       </x:c>
       <x:c r="K212" s="13" t="str">
-        <x:v>待完成</x:v>
+        <x:v>已完成</x:v>
       </x:c>
       <x:c r="L212" s="13" t="str">
         <x:v>09-08～09-10</x:v>
       </x:c>
       <x:c r="M212" s="13" t="str">
-        <x:v>—</x:v>
+        <x:v>2026-08-21</x:v>
       </x:c>
       <x:c r="N212" s="13" t="str">
         <x:v>job/variant/asset UUID；archive_id UUID；归档键=用户+选择集+尺寸</x:v>
@@ -12413,13 +12413,13 @@
         <x:v>FE-ZIP-02</x:v>
       </x:c>
       <x:c r="K213" s="13" t="str">
-        <x:v>待完成</x:v>
+        <x:v>已完成</x:v>
       </x:c>
       <x:c r="L213" s="13" t="str">
         <x:v>09-08～09-10</x:v>
       </x:c>
       <x:c r="M213" s="13" t="str">
-        <x:v>—</x:v>
+        <x:v>2026-08-21</x:v>
       </x:c>
       <x:c r="N213" s="13" t="str">
         <x:v>job/variant/asset UUID；archive_id UUID；归档键=用户+选择集+尺寸</x:v>
@@ -12469,13 +12469,13 @@
         <x:v>FE-ZIP-02</x:v>
       </x:c>
       <x:c r="K214" s="13" t="str">
-        <x:v>待完成</x:v>
+        <x:v>已完成</x:v>
       </x:c>
       <x:c r="L214" s="13" t="str">
         <x:v>09-08～09-10</x:v>
       </x:c>
       <x:c r="M214" s="13" t="str">
-        <x:v>—</x:v>
+        <x:v>2026-08-21</x:v>
       </x:c>
       <x:c r="N214" s="13" t="str">
         <x:v>job/variant/asset UUID；archive_id UUID；归档键=用户+选择集+尺寸</x:v>
@@ -12525,13 +12525,13 @@
         <x:v>—</x:v>
       </x:c>
       <x:c r="K215" s="13" t="str">
-        <x:v>待完成</x:v>
+        <x:v>已完成</x:v>
       </x:c>
       <x:c r="L215" s="13" t="str">
         <x:v>09-08～09-10</x:v>
       </x:c>
       <x:c r="M215" s="13" t="str">
-        <x:v>—</x:v>
+        <x:v>2026-08-21</x:v>
       </x:c>
       <x:c r="N215" s="13" t="str">
         <x:v>job/variant/asset UUID；archive_id UUID；归档键=用户+选择集+尺寸</x:v>
@@ -15085,7 +15085,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R09168eb1542b4458"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R3e3635cbdb9e4703"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -16776,7 +16776,7 @@
         <x:v>GEN-004/005</x:v>
       </x:c>
       <x:c r="D32" s="13" t="str">
-        <x:v>核心设置API</x:v>
+        <x:v>图标设计风格API</x:v>
       </x:c>
       <x:c r="E32" s="13" t="str">
         <x:v>BE-SETTINGS-01</x:v>
@@ -16785,7 +16785,7 @@
         <x:v>后端</x:v>
       </x:c>
       <x:c r="G32" s="13" t="str">
-        <x:v>定义GET /api/generation/settings请求响应契约</x:v>
+        <x:v>定义GET /api/generation/settings风格契约</x:v>
       </x:c>
       <x:c r="H32" s="13" t="str">
         <x:v>共享Schema、类型和示例</x:v>
@@ -16803,7 +16803,7 @@
         <x:v>08-22</x:v>
       </x:c>
       <x:c r="M32" s="13" t="str">
-        <x:v>2026-08-20</x:v>
+        <x:v>2026-08-22</x:v>
       </x:c>
       <x:c r="N32" s="13" t="str">
         <x:v>job/subject/variant/asset均为UUID；创建请求带idempotency_key；记录设置/Skill/模型版本</x:v>
@@ -16832,7 +16832,7 @@
         <x:v>GEN-004/005</x:v>
       </x:c>
       <x:c r="D33" s="13" t="str">
-        <x:v>核心设置API</x:v>
+        <x:v>图标设计风格API</x:v>
       </x:c>
       <x:c r="E33" s="13" t="str">
         <x:v>BE-SETTINGS-02</x:v>
@@ -16859,7 +16859,7 @@
         <x:v>08-22</x:v>
       </x:c>
       <x:c r="M33" s="13" t="str">
-        <x:v>2026-08-20</x:v>
+        <x:v>2026-08-22</x:v>
       </x:c>
       <x:c r="N33" s="13" t="str">
         <x:v>job/subject/variant/asset均为UUID；创建请求带idempotency_key；记录设置/Skill/模型版本</x:v>
@@ -16888,7 +16888,7 @@
         <x:v>GEN-004/005</x:v>
       </x:c>
       <x:c r="D34" s="13" t="str">
-        <x:v>核心设置API</x:v>
+        <x:v>图标设计风格API</x:v>
       </x:c>
       <x:c r="E34" s="13" t="str">
         <x:v>BE-SETTINGS-03</x:v>
@@ -16915,7 +16915,7 @@
         <x:v>08-22</x:v>
       </x:c>
       <x:c r="M34" s="13" t="str">
-        <x:v>2026-08-20</x:v>
+        <x:v>2026-08-22</x:v>
       </x:c>
       <x:c r="N34" s="13" t="str">
         <x:v>job/subject/variant/asset均为UUID；创建请求带idempotency_key；记录设置/Skill/模型版本</x:v>
@@ -16944,7 +16944,7 @@
         <x:v>GEN-004/005</x:v>
       </x:c>
       <x:c r="D35" s="13" t="str">
-        <x:v>核心设置API</x:v>
+        <x:v>图标设计风格API</x:v>
       </x:c>
       <x:c r="E35" s="13" t="str">
         <x:v>BE-SETTINGS-04</x:v>
@@ -16953,7 +16953,7 @@
         <x:v>后端</x:v>
       </x:c>
       <x:c r="G35" s="13" t="str">
-        <x:v>返回设置版本</x:v>
+        <x:v>返回图标设计风格版本</x:v>
       </x:c>
       <x:c r="H35" s="13" t="str">
         <x:v>settingsVersion字段</x:v>
@@ -16971,7 +16971,7 @@
         <x:v>08-22</x:v>
       </x:c>
       <x:c r="M35" s="13" t="str">
-        <x:v>2026-08-20</x:v>
+        <x:v>2026-08-22</x:v>
       </x:c>
       <x:c r="N35" s="13" t="str">
         <x:v>job/subject/variant/asset均为UUID；创建请求带idempotency_key；记录设置/Skill/模型版本</x:v>
@@ -17000,7 +17000,7 @@
         <x:v>GEN-004/005</x:v>
       </x:c>
       <x:c r="D36" s="13" t="str">
-        <x:v>核心设置API</x:v>
+        <x:v>图标设计风格API</x:v>
       </x:c>
       <x:c r="E36" s="13" t="str">
         <x:v>BE-SETTINGS-05</x:v>
@@ -17009,13 +17009,13 @@
         <x:v>后端</x:v>
       </x:c>
       <x:c r="G36" s="13" t="str">
-        <x:v>返回6组25项</x:v>
+        <x:v>返回5个预设与3组微调</x:v>
       </x:c>
       <x:c r="H36" s="13" t="str">
-        <x:v>稳定ID、en/zh label、prompt token</x:v>
+        <x:v>稳定ID、en/zh label、description、prompt token</x:v>
       </x:c>
       <x:c r="I36" s="13" t="str">
-        <x:v>自动测试数量和重复ID</x:v>
+        <x:v>自动测试预设、微调组和重复ID</x:v>
       </x:c>
       <x:c r="J36" s="13" t="str">
         <x:v>—</x:v>
@@ -17027,7 +17027,7 @@
         <x:v>08-22</x:v>
       </x:c>
       <x:c r="M36" s="13" t="str">
-        <x:v>2026-08-20</x:v>
+        <x:v>2026-08-22</x:v>
       </x:c>
       <x:c r="N36" s="13" t="str">
         <x:v>job/subject/variant/asset均为UUID；创建请求带idempotency_key；记录设置/Skill/模型版本</x:v>
@@ -17056,7 +17056,7 @@
         <x:v>GEN-004/005</x:v>
       </x:c>
       <x:c r="D37" s="13" t="str">
-        <x:v>核心设置API</x:v>
+        <x:v>图标设计风格API</x:v>
       </x:c>
       <x:c r="E37" s="13" t="str">
         <x:v>BE-SETTINGS-06</x:v>
@@ -17065,13 +17065,13 @@
         <x:v>后端</x:v>
       </x:c>
       <x:c r="G37" s="13" t="str">
-        <x:v>返回允许尺寸和主体上限</x:v>
+        <x:v>返回允许尺寸和生成规则</x:v>
       </x:c>
       <x:c r="H37" s="13" t="str">
-        <x:v>sizes/maxSubjects/variantsPerSubject</x:v>
+        <x:v>sizes/maxOutputSizes/variantsPerSubject</x:v>
       </x:c>
       <x:c r="I37" s="13" t="str">
-        <x:v>数值来自共享常量</x:v>
+        <x:v>数值来自共享常量；不返回主体上限</x:v>
       </x:c>
       <x:c r="J37" s="13" t="str">
         <x:v>—</x:v>
@@ -17083,7 +17083,7 @@
         <x:v>08-22</x:v>
       </x:c>
       <x:c r="M37" s="13" t="str">
-        <x:v>2026-08-20</x:v>
+        <x:v>2026-08-22</x:v>
       </x:c>
       <x:c r="N37" s="13" t="str">
         <x:v>job/subject/variant/asset均为UUID；创建请求带idempotency_key；记录设置/Skill/模型版本</x:v>
@@ -17112,7 +17112,7 @@
         <x:v>GEN-004/005</x:v>
       </x:c>
       <x:c r="D38" s="13" t="str">
-        <x:v>核心设置API</x:v>
+        <x:v>图标设计风格API</x:v>
       </x:c>
       <x:c r="E38" s="13" t="str">
         <x:v>BE-SETTINGS-07</x:v>
@@ -17139,7 +17139,7 @@
         <x:v>08-22</x:v>
       </x:c>
       <x:c r="M38" s="13" t="str">
-        <x:v>2026-08-20</x:v>
+        <x:v>2026-08-22</x:v>
       </x:c>
       <x:c r="N38" s="13" t="str">
         <x:v>job/subject/variant/asset均为UUID；创建请求带idempotency_key；记录设置/Skill/模型版本</x:v>
@@ -17168,7 +17168,7 @@
         <x:v>GEN-004/005</x:v>
       </x:c>
       <x:c r="D39" s="13" t="str">
-        <x:v>核心设置API</x:v>
+        <x:v>图标设计风格API</x:v>
       </x:c>
       <x:c r="E39" s="13" t="str">
         <x:v>BE-SETTINGS-08</x:v>
@@ -17177,7 +17177,7 @@
         <x:v>后端</x:v>
       </x:c>
       <x:c r="G39" s="13" t="str">
-        <x:v>编写GET /api/generation/settings单元与集成测试</x:v>
+        <x:v>编写图标设计风格设置接口测试</x:v>
       </x:c>
       <x:c r="H39" s="13" t="str">
         <x:v>Schema、数量、缓存和重复调用测试</x:v>
@@ -17195,7 +17195,7 @@
         <x:v>08-22</x:v>
       </x:c>
       <x:c r="M39" s="13" t="str">
-        <x:v>2026-08-20</x:v>
+        <x:v>2026-08-22</x:v>
       </x:c>
       <x:c r="N39" s="13" t="str">
         <x:v>job/subject/variant/asset均为UUID；创建请求带idempotency_key；记录设置/Skill/模型版本</x:v>
@@ -17224,7 +17224,7 @@
         <x:v>GEN-004/005</x:v>
       </x:c>
       <x:c r="D40" s="13" t="str">
-        <x:v>核心设置API</x:v>
+        <x:v>图标设计风格API</x:v>
       </x:c>
       <x:c r="E40" s="13" t="str">
         <x:v>BE-SETTINGS-09</x:v>
@@ -17233,7 +17233,7 @@
         <x:v>后端</x:v>
       </x:c>
       <x:c r="G40" s="13" t="str">
-        <x:v>更新GET /api/generation/settings接口文档</x:v>
+        <x:v>更新图标设计风格设置接口文档</x:v>
       </x:c>
       <x:c r="H40" s="13" t="str">
         <x:v>请求、响应、错误、鉴权和示例</x:v>
@@ -17251,7 +17251,7 @@
         <x:v>08-22</x:v>
       </x:c>
       <x:c r="M40" s="13" t="str">
-        <x:v>2026-08-20</x:v>
+        <x:v>2026-08-22</x:v>
       </x:c>
       <x:c r="N40" s="13" t="str">
         <x:v>job/subject/variant/asset均为UUID；创建请求带idempotency_key；记录设置/Skill/模型版本</x:v>
@@ -17301,13 +17301,13 @@
         <x:v>—</x:v>
       </x:c>
       <x:c r="K41" s="13" t="str">
-        <x:v>待完成</x:v>
+        <x:v>已完成</x:v>
       </x:c>
       <x:c r="L41" s="13" t="str">
         <x:v>08-22～08-24</x:v>
       </x:c>
       <x:c r="M41" s="13" t="str">
-        <x:v>—</x:v>
+        <x:v>2026-08-21</x:v>
       </x:c>
       <x:c r="N41" s="13" t="str">
         <x:v>job/subject/variant/asset均为UUID；创建请求带idempotency_key；记录设置/Skill/模型版本</x:v>
@@ -17345,25 +17345,25 @@
         <x:v>后端</x:v>
       </x:c>
       <x:c r="G42" s="13" t="str">
-        <x:v>实现POST /api/generation/jobs输入校验</x:v>
+        <x:v>校验POST /api/generation/jobs风格输入</x:v>
       </x:c>
       <x:c r="H42" s="13" t="str">
-        <x:v>边界校验与字段规范化</x:v>
+        <x:v>主体、style和尺寸校验</x:v>
       </x:c>
       <x:c r="I42" s="13" t="str">
-        <x:v>非法输入在副作用前返回稳定400错误</x:v>
+        <x:v>非法风格在数据库副作用前返回稳定400错误</x:v>
       </x:c>
       <x:c r="J42" s="13" t="str">
         <x:v>BE-JOB-CREATE-01</x:v>
       </x:c>
       <x:c r="K42" s="13" t="str">
-        <x:v>待完成</x:v>
+        <x:v>已完成</x:v>
       </x:c>
       <x:c r="L42" s="13" t="str">
         <x:v>08-22～08-24</x:v>
       </x:c>
       <x:c r="M42" s="13" t="str">
-        <x:v>—</x:v>
+        <x:v>2026-08-22</x:v>
       </x:c>
       <x:c r="N42" s="13" t="str">
         <x:v>job/subject/variant/asset均为UUID；创建请求带idempotency_key；记录设置/Skill/模型版本</x:v>
@@ -17413,13 +17413,13 @@
         <x:v>BE-JOB-CREATE-01</x:v>
       </x:c>
       <x:c r="K43" s="13" t="str">
-        <x:v>待完成</x:v>
+        <x:v>已完成</x:v>
       </x:c>
       <x:c r="L43" s="13" t="str">
         <x:v>08-22～08-24</x:v>
       </x:c>
       <x:c r="M43" s="13" t="str">
-        <x:v>—</x:v>
+        <x:v>2026-08-21</x:v>
       </x:c>
       <x:c r="N43" s="13" t="str">
         <x:v>job/subject/variant/asset均为UUID；创建请求带idempotency_key；记录设置/Skill/模型版本</x:v>
@@ -17457,7 +17457,7 @@
         <x:v>后端</x:v>
       </x:c>
       <x:c r="G44" s="13" t="str">
-        <x:v>校验设置版本</x:v>
+        <x:v>校验图标设计风格版本</x:v>
       </x:c>
       <x:c r="H44" s="13" t="str">
         <x:v>拒绝过期settingsVersion</x:v>
@@ -17469,13 +17469,13 @@
         <x:v>—</x:v>
       </x:c>
       <x:c r="K44" s="13" t="str">
-        <x:v>待完成</x:v>
+        <x:v>已完成</x:v>
       </x:c>
       <x:c r="L44" s="13" t="str">
         <x:v>08-22～08-24</x:v>
       </x:c>
       <x:c r="M44" s="13" t="str">
-        <x:v>—</x:v>
+        <x:v>2026-08-22</x:v>
       </x:c>
       <x:c r="N44" s="13" t="str">
         <x:v>job/subject/variant/asset均为UUID；创建请求带idempotency_key；记录设置/Skill/模型版本</x:v>
@@ -17513,25 +17513,25 @@
         <x:v>后端</x:v>
       </x:c>
       <x:c r="G45" s="13" t="str">
-        <x:v>校验1–20主体与唯一clientId</x:v>
+        <x:v>校验主体与唯一clientId</x:v>
       </x:c>
       <x:c r="H45" s="13" t="str">
         <x:v>Schema和数据库双层约束</x:v>
       </x:c>
       <x:c r="I45" s="13" t="str">
-        <x:v>无效请求不扣点</x:v>
+        <x:v>不限制20个主体；无效请求不创建任务</x:v>
       </x:c>
       <x:c r="J45" s="13" t="str">
         <x:v>—</x:v>
       </x:c>
       <x:c r="K45" s="13" t="str">
-        <x:v>待完成</x:v>
+        <x:v>已完成</x:v>
       </x:c>
       <x:c r="L45" s="13" t="str">
         <x:v>08-22～08-24</x:v>
       </x:c>
       <x:c r="M45" s="13" t="str">
-        <x:v>—</x:v>
+        <x:v>2026-08-21</x:v>
       </x:c>
       <x:c r="N45" s="13" t="str">
         <x:v>job/subject/variant/asset均为UUID；创建请求带idempotency_key；记录设置/Skill/模型版本</x:v>
@@ -17575,7 +17575,7 @@
         <x:v>主体名称和描述安全检查</x:v>
       </x:c>
       <x:c r="I46" s="13" t="str">
-        <x:v>拦截请求不扣点</x:v>
+        <x:v>拦截请求不进入生成队列</x:v>
       </x:c>
       <x:c r="J46" s="13" t="str">
         <x:v>—</x:v>
@@ -17637,13 +17637,13 @@
         <x:v>—</x:v>
       </x:c>
       <x:c r="K47" s="13" t="str">
-        <x:v>待完成</x:v>
+        <x:v>已完成</x:v>
       </x:c>
       <x:c r="L47" s="13" t="str">
         <x:v>08-22～08-24</x:v>
       </x:c>
       <x:c r="M47" s="13" t="str">
-        <x:v>—</x:v>
+        <x:v>2026-08-21</x:v>
       </x:c>
       <x:c r="N47" s="13" t="str">
         <x:v>job/subject/variant/asset均为UUID；创建请求带idempotency_key；记录设置/Skill/模型版本</x:v>
@@ -17681,25 +17681,25 @@
         <x:v>后端</x:v>
       </x:c>
       <x:c r="G48" s="13" t="str">
-        <x:v>锁定点数账户</x:v>
+        <x:v>校验活动任务并发边界</x:v>
       </x:c>
       <x:c r="H48" s="13" t="str">
-        <x:v>SELECT FOR UPDATE</x:v>
+        <x:v>同一用户queued/processing任务限制</x:v>
       </x:c>
       <x:c r="I48" s="13" t="str">
-        <x:v>并发提交不会透支</x:v>
+        <x:v>并发请求不创建重复活动任务</x:v>
       </x:c>
       <x:c r="J48" s="13" t="str">
         <x:v>—</x:v>
       </x:c>
       <x:c r="K48" s="13" t="str">
-        <x:v>待完成</x:v>
+        <x:v>已完成</x:v>
       </x:c>
       <x:c r="L48" s="13" t="str">
         <x:v>08-22～08-24</x:v>
       </x:c>
       <x:c r="M48" s="13" t="str">
-        <x:v>—</x:v>
+        <x:v>2026-08-21</x:v>
       </x:c>
       <x:c r="N48" s="13" t="str">
         <x:v>job/subject/variant/asset均为UUID；创建请求带idempotency_key；记录设置/Skill/模型版本</x:v>
@@ -17737,25 +17737,25 @@
         <x:v>后端</x:v>
       </x:c>
       <x:c r="G49" s="13" t="str">
-        <x:v>计算服务端费用</x:v>
+        <x:v>规范化生成规格快照</x:v>
       </x:c>
       <x:c r="H49" s="13" t="str">
-        <x:v>subject count×1</x:v>
+        <x:v>主体、颜色、背景、style与尺寸</x:v>
       </x:c>
       <x:c r="I49" s="13" t="str">
-        <x:v>忽略客户端费用</x:v>
+        <x:v>生成任务不接收或计算点数字段</x:v>
       </x:c>
       <x:c r="J49" s="13" t="str">
         <x:v>—</x:v>
       </x:c>
       <x:c r="K49" s="13" t="str">
-        <x:v>待完成</x:v>
+        <x:v>已完成</x:v>
       </x:c>
       <x:c r="L49" s="13" t="str">
         <x:v>08-22～08-24</x:v>
       </x:c>
       <x:c r="M49" s="13" t="str">
-        <x:v>—</x:v>
+        <x:v>2026-08-22</x:v>
       </x:c>
       <x:c r="N49" s="13" t="str">
         <x:v>job/subject/variant/asset均为UUID；创建请求带idempotency_key；记录设置/Skill/模型版本</x:v>
@@ -17805,13 +17805,13 @@
         <x:v>—</x:v>
       </x:c>
       <x:c r="K50" s="13" t="str">
-        <x:v>待完成</x:v>
+        <x:v>已完成</x:v>
       </x:c>
       <x:c r="L50" s="13" t="str">
         <x:v>08-22～08-24</x:v>
       </x:c>
       <x:c r="M50" s="13" t="str">
-        <x:v>—</x:v>
+        <x:v>2026-08-21</x:v>
       </x:c>
       <x:c r="N50" s="13" t="str">
         <x:v>job/subject/variant/asset均为UUID；创建请求带idempotency_key；记录设置/Skill/模型版本</x:v>
@@ -17849,25 +17849,25 @@
         <x:v>后端</x:v>
       </x:c>
       <x:c r="G51" s="13" t="str">
-        <x:v>原子扣点并写账本</x:v>
+        <x:v>原子写入生成任务关联数据</x:v>
       </x:c>
       <x:c r="H51" s="13" t="str">
-        <x:v>generation_debit和balance_after</x:v>
+        <x:v>job、subjects与每主体3个variants</x:v>
       </x:c>
       <x:c r="I51" s="13" t="str">
-        <x:v>与任务使用同一事务</x:v>
+        <x:v>任一写入失败全部回滚；不操作点数账本</x:v>
       </x:c>
       <x:c r="J51" s="13" t="str">
         <x:v>—</x:v>
       </x:c>
       <x:c r="K51" s="13" t="str">
-        <x:v>待完成</x:v>
+        <x:v>已完成</x:v>
       </x:c>
       <x:c r="L51" s="13" t="str">
         <x:v>08-22～08-24</x:v>
       </x:c>
       <x:c r="M51" s="13" t="str">
-        <x:v>—</x:v>
+        <x:v>2026-08-21</x:v>
       </x:c>
       <x:c r="N51" s="13" t="str">
         <x:v>job/subject/variant/asset均为UUID；创建请求带idempotency_key；记录设置/Skill/模型版本</x:v>
@@ -17908,22 +17908,22 @@
         <x:v>写入创建幂等键</x:v>
       </x:c>
       <x:c r="H52" s="13" t="str">
-        <x:v>idempotencyKey唯一</x:v>
+        <x:v>generation_jobs(user_id,idempotency_key)唯一</x:v>
       </x:c>
       <x:c r="I52" s="13" t="str">
-        <x:v>重复请求返回原job且不再次扣点</x:v>
+        <x:v>重复请求返回原job且不创建第二任务</x:v>
       </x:c>
       <x:c r="J52" s="13" t="str">
         <x:v>—</x:v>
       </x:c>
       <x:c r="K52" s="13" t="str">
-        <x:v>待完成</x:v>
+        <x:v>已完成</x:v>
       </x:c>
       <x:c r="L52" s="13" t="str">
         <x:v>08-22～08-24</x:v>
       </x:c>
       <x:c r="M52" s="13" t="str">
-        <x:v>—</x:v>
+        <x:v>2026-08-21</x:v>
       </x:c>
       <x:c r="N52" s="13" t="str">
         <x:v>job/subject/variant/asset均为UUID；创建请求带idempotency_key；记录设置/Skill/模型版本</x:v>
@@ -18029,13 +18029,13 @@
         <x:v>BE-JOB-CREATE-02</x:v>
       </x:c>
       <x:c r="K54" s="13" t="str">
-        <x:v>待完成</x:v>
+        <x:v>已完成</x:v>
       </x:c>
       <x:c r="L54" s="13" t="str">
         <x:v>08-22～08-24</x:v>
       </x:c>
       <x:c r="M54" s="13" t="str">
-        <x:v>—</x:v>
+        <x:v>2026-08-21</x:v>
       </x:c>
       <x:c r="N54" s="13" t="str">
         <x:v>job/subject/variant/asset均为UUID；创建请求带idempotency_key；记录设置/Skill/模型版本</x:v>
@@ -18197,13 +18197,13 @@
         <x:v>—</x:v>
       </x:c>
       <x:c r="K57" s="13" t="str">
-        <x:v>待完成</x:v>
+        <x:v>已完成</x:v>
       </x:c>
       <x:c r="L57" s="13" t="str">
         <x:v>08-25～08-26</x:v>
       </x:c>
       <x:c r="M57" s="13" t="str">
-        <x:v>—</x:v>
+        <x:v>2026-08-21</x:v>
       </x:c>
       <x:c r="N57" s="13" t="str">
         <x:v>job/subject/variant/asset均为UUID；创建请求带idempotency_key；记录设置/Skill/模型版本</x:v>
@@ -18253,13 +18253,13 @@
         <x:v>BE-JOB-QUERY-01</x:v>
       </x:c>
       <x:c r="K58" s="13" t="str">
-        <x:v>待完成</x:v>
+        <x:v>已完成</x:v>
       </x:c>
       <x:c r="L58" s="13" t="str">
         <x:v>08-25～08-26</x:v>
       </x:c>
       <x:c r="M58" s="13" t="str">
-        <x:v>—</x:v>
+        <x:v>2026-08-21</x:v>
       </x:c>
       <x:c r="N58" s="13" t="str">
         <x:v>job/subject/variant/asset均为UUID；创建请求带idempotency_key；记录设置/Skill/模型版本</x:v>
@@ -18309,13 +18309,13 @@
         <x:v>BE-JOB-QUERY-01</x:v>
       </x:c>
       <x:c r="K59" s="13" t="str">
-        <x:v>待完成</x:v>
+        <x:v>已完成</x:v>
       </x:c>
       <x:c r="L59" s="13" t="str">
         <x:v>08-25～08-26</x:v>
       </x:c>
       <x:c r="M59" s="13" t="str">
-        <x:v>—</x:v>
+        <x:v>2026-08-21</x:v>
       </x:c>
       <x:c r="N59" s="13" t="str">
         <x:v>job/subject/variant/asset均为UUID；创建请求带idempotency_key；记录设置/Skill/模型版本</x:v>
@@ -18365,13 +18365,13 @@
         <x:v>—</x:v>
       </x:c>
       <x:c r="K60" s="13" t="str">
-        <x:v>待完成</x:v>
+        <x:v>已完成</x:v>
       </x:c>
       <x:c r="L60" s="13" t="str">
         <x:v>08-25～08-26</x:v>
       </x:c>
       <x:c r="M60" s="13" t="str">
-        <x:v>—</x:v>
+        <x:v>2026-08-21</x:v>
       </x:c>
       <x:c r="N60" s="13" t="str">
         <x:v>job/subject/variant/asset均为UUID；创建请求带idempotency_key；记录设置/Skill/模型版本</x:v>
@@ -18421,13 +18421,13 @@
         <x:v>—</x:v>
       </x:c>
       <x:c r="K61" s="13" t="str">
-        <x:v>待完成</x:v>
+        <x:v>已完成</x:v>
       </x:c>
       <x:c r="L61" s="13" t="str">
         <x:v>08-25～08-26</x:v>
       </x:c>
       <x:c r="M61" s="13" t="str">
-        <x:v>—</x:v>
+        <x:v>2026-08-21</x:v>
       </x:c>
       <x:c r="N61" s="13" t="str">
         <x:v>job/subject/variant/asset均为UUID；创建请求带idempotency_key；记录设置/Skill/模型版本</x:v>
@@ -18477,13 +18477,13 @@
         <x:v>—</x:v>
       </x:c>
       <x:c r="K62" s="13" t="str">
-        <x:v>待完成</x:v>
+        <x:v>已完成</x:v>
       </x:c>
       <x:c r="L62" s="13" t="str">
         <x:v>08-25～08-26</x:v>
       </x:c>
       <x:c r="M62" s="13" t="str">
-        <x:v>—</x:v>
+        <x:v>2026-08-21</x:v>
       </x:c>
       <x:c r="N62" s="13" t="str">
         <x:v>job/subject/variant/asset均为UUID；创建请求带idempotency_key；记录设置/Skill/模型版本</x:v>
@@ -18533,13 +18533,13 @@
         <x:v>—</x:v>
       </x:c>
       <x:c r="K63" s="13" t="str">
-        <x:v>待完成</x:v>
+        <x:v>已完成</x:v>
       </x:c>
       <x:c r="L63" s="13" t="str">
         <x:v>08-25～08-26</x:v>
       </x:c>
       <x:c r="M63" s="13" t="str">
-        <x:v>—</x:v>
+        <x:v>2026-08-21</x:v>
       </x:c>
       <x:c r="N63" s="13" t="str">
         <x:v>job/subject/variant/asset均为UUID；创建请求带idempotency_key；记录设置/Skill/模型版本</x:v>
@@ -18577,25 +18577,25 @@
         <x:v>后端</x:v>
       </x:c>
       <x:c r="G64" s="13" t="str">
-        <x:v>返回扣点返还摘要</x:v>
+        <x:v>返回当前处理主体</x:v>
       </x:c>
       <x:c r="H64" s="13" t="str">
-        <x:v>charged/refunded</x:v>
+        <x:v>currentSubjectName与completedSubjects</x:v>
       </x:c>
       <x:c r="I64" s="13" t="str">
-        <x:v>与账本聚合一致</x:v>
+        <x:v>进度文本可直接由前端本地化，不返回点数摘要</x:v>
       </x:c>
       <x:c r="J64" s="13" t="str">
         <x:v>—</x:v>
       </x:c>
       <x:c r="K64" s="13" t="str">
-        <x:v>待完成</x:v>
+        <x:v>已完成</x:v>
       </x:c>
       <x:c r="L64" s="13" t="str">
         <x:v>08-25～08-26</x:v>
       </x:c>
       <x:c r="M64" s="13" t="str">
-        <x:v>—</x:v>
+        <x:v>2026-08-21</x:v>
       </x:c>
       <x:c r="N64" s="13" t="str">
         <x:v>job/subject/variant/asset均为UUID；创建请求带idempotency_key；记录设置/Skill/模型版本</x:v>
@@ -18645,13 +18645,13 @@
         <x:v>BE-JOB-QUERY-02</x:v>
       </x:c>
       <x:c r="K65" s="13" t="str">
-        <x:v>待完成</x:v>
+        <x:v>已完成</x:v>
       </x:c>
       <x:c r="L65" s="13" t="str">
         <x:v>08-25～08-26</x:v>
       </x:c>
       <x:c r="M65" s="13" t="str">
-        <x:v>—</x:v>
+        <x:v>2026-08-21</x:v>
       </x:c>
       <x:c r="N65" s="13" t="str">
         <x:v>job/subject/variant/asset均为UUID；创建请求带idempotency_key；记录设置/Skill/模型版本</x:v>
@@ -19081,13 +19081,13 @@
         <x:v>后端</x:v>
       </x:c>
       <x:c r="G73" s="13" t="str">
-        <x:v>编译主体提示词</x:v>
+        <x:v>编译主体图标设计风格提示词</x:v>
       </x:c>
       <x:c r="H73" s="13" t="str">
-        <x:v>主体+颜色+背景+25项+slot</x:v>
+        <x:v>主体+颜色+背景+style+slot</x:v>
       </x:c>
       <x:c r="I73" s="13" t="str">
-        <x:v>不生成App Store图标</x:v>
+        <x:v>不生成App Store图标；批次统一使用同一风格</x:v>
       </x:c>
       <x:c r="J73" s="13" t="str">
         <x:v>—</x:v>
@@ -19099,7 +19099,7 @@
         <x:v>08-23～08-25</x:v>
       </x:c>
       <x:c r="M73" s="13" t="str">
-        <x:v>2026-08-20</x:v>
+        <x:v>2026-08-22</x:v>
       </x:c>
       <x:c r="N73" s="13" t="str">
         <x:v>job/subject/variant/asset均为UUID；创建请求带idempotency_key；记录设置/Skill/模型版本</x:v>
@@ -19529,13 +19529,13 @@
         <x:v>后端</x:v>
       </x:c>
       <x:c r="G81" s="13" t="str">
-        <x:v>生成批次一致性约束</x:v>
+        <x:v>生成批次设计风格一致性约束</x:v>
       </x:c>
       <x:c r="H81" s="13" t="str">
-        <x:v>统一结构/笔触/颜色/视角</x:v>
+        <x:v>预设、线条、转角、细节、颜色与视角约束</x:v>
       </x:c>
       <x:c r="I81" s="13" t="str">
-        <x:v>同批主体保持一致视觉语言</x:v>
+        <x:v>同批主体保持一致图标设计风格</x:v>
       </x:c>
       <x:c r="J81" s="13" t="str">
         <x:v>—</x:v>
@@ -19547,7 +19547,7 @@
         <x:v>08-23～08-25</x:v>
       </x:c>
       <x:c r="M81" s="13" t="str">
-        <x:v>2026-08-20</x:v>
+        <x:v>2026-08-22</x:v>
       </x:c>
       <x:c r="N81" s="13" t="str">
         <x:v>job/subject/variant/asset均为UUID；创建请求带idempotency_key；记录设置/Skill/模型版本</x:v>
@@ -20145,13 +20145,13 @@
         <x:v>后端</x:v>
       </x:c>
       <x:c r="G92" s="13" t="str">
-        <x:v>在扣点前检查请求</x:v>
+        <x:v>在创建任务前检查请求</x:v>
       </x:c>
       <x:c r="H92" s="13" t="str">
         <x:v>内容分类服务</x:v>
       </x:c>
       <x:c r="I92" s="13" t="str">
-        <x:v>拦截不创建任务不扣点</x:v>
+        <x:v>拦截请求不进入任务队列；与点数模块解耦</x:v>
       </x:c>
       <x:c r="J92" s="13" t="str">
         <x:v>—</x:v>
@@ -21445,13 +21445,13 @@
         <x:v>—</x:v>
       </x:c>
       <x:c r="K115" s="13" t="str">
-        <x:v>待完成</x:v>
+        <x:v>已完成</x:v>
       </x:c>
       <x:c r="L115" s="13" t="str">
         <x:v>09-04～09-06</x:v>
       </x:c>
       <x:c r="M115" s="13" t="str">
-        <x:v>—</x:v>
+        <x:v>2026-08-21</x:v>
       </x:c>
       <x:c r="N115" s="13" t="str">
         <x:v>job/variant/asset UUID；archive_id UUID；归档键=用户+选择集+尺寸</x:v>
@@ -21501,13 +21501,13 @@
         <x:v>BE-PRIMARY-01</x:v>
       </x:c>
       <x:c r="K116" s="13" t="str">
-        <x:v>待完成</x:v>
+        <x:v>已完成</x:v>
       </x:c>
       <x:c r="L116" s="13" t="str">
         <x:v>09-04～09-06</x:v>
       </x:c>
       <x:c r="M116" s="13" t="str">
-        <x:v>—</x:v>
+        <x:v>2026-08-21</x:v>
       </x:c>
       <x:c r="N116" s="13" t="str">
         <x:v>job/variant/asset UUID；archive_id UUID；归档键=用户+选择集+尺寸</x:v>
@@ -21557,13 +21557,13 @@
         <x:v>BE-PRIMARY-01</x:v>
       </x:c>
       <x:c r="K117" s="13" t="str">
-        <x:v>待完成</x:v>
+        <x:v>已完成</x:v>
       </x:c>
       <x:c r="L117" s="13" t="str">
         <x:v>09-04～09-06</x:v>
       </x:c>
       <x:c r="M117" s="13" t="str">
-        <x:v>—</x:v>
+        <x:v>2026-08-21</x:v>
       </x:c>
       <x:c r="N117" s="13" t="str">
         <x:v>job/variant/asset UUID；archive_id UUID；归档键=用户+选择集+尺寸</x:v>
@@ -21613,13 +21613,13 @@
         <x:v>—</x:v>
       </x:c>
       <x:c r="K118" s="13" t="str">
-        <x:v>待完成</x:v>
+        <x:v>已完成</x:v>
       </x:c>
       <x:c r="L118" s="13" t="str">
         <x:v>09-04～09-06</x:v>
       </x:c>
       <x:c r="M118" s="13" t="str">
-        <x:v>—</x:v>
+        <x:v>2026-08-21</x:v>
       </x:c>
       <x:c r="N118" s="13" t="str">
         <x:v>job/variant/asset UUID；archive_id UUID；归档键=用户+选择集+尺寸</x:v>
@@ -21669,13 +21669,13 @@
         <x:v>—</x:v>
       </x:c>
       <x:c r="K119" s="13" t="str">
-        <x:v>待完成</x:v>
+        <x:v>已完成</x:v>
       </x:c>
       <x:c r="L119" s="13" t="str">
         <x:v>09-04～09-06</x:v>
       </x:c>
       <x:c r="M119" s="13" t="str">
-        <x:v>—</x:v>
+        <x:v>2026-08-21</x:v>
       </x:c>
       <x:c r="N119" s="13" t="str">
         <x:v>job/variant/asset UUID；archive_id UUID；归档键=用户+选择集+尺寸</x:v>
@@ -21725,13 +21725,13 @@
         <x:v>—</x:v>
       </x:c>
       <x:c r="K120" s="13" t="str">
-        <x:v>待完成</x:v>
+        <x:v>已完成</x:v>
       </x:c>
       <x:c r="L120" s="13" t="str">
         <x:v>09-04～09-06</x:v>
       </x:c>
       <x:c r="M120" s="13" t="str">
-        <x:v>—</x:v>
+        <x:v>2026-08-21</x:v>
       </x:c>
       <x:c r="N120" s="13" t="str">
         <x:v>job/variant/asset UUID；archive_id UUID；归档键=用户+选择集+尺寸</x:v>
@@ -21781,13 +21781,13 @@
         <x:v>BE-PRIMARY-02</x:v>
       </x:c>
       <x:c r="K121" s="13" t="str">
-        <x:v>待完成</x:v>
+        <x:v>已完成</x:v>
       </x:c>
       <x:c r="L121" s="13" t="str">
         <x:v>09-04～09-06</x:v>
       </x:c>
       <x:c r="M121" s="13" t="str">
-        <x:v>—</x:v>
+        <x:v>2026-08-21</x:v>
       </x:c>
       <x:c r="N121" s="13" t="str">
         <x:v>job/variant/asset UUID；archive_id UUID；归档键=用户+选择集+尺寸</x:v>
@@ -22497,25 +22497,25 @@
         <x:v>后端</x:v>
       </x:c>
       <x:c r="G134" s="13" t="str">
-        <x:v>定义POST/GET downloads请求响应契约</x:v>
+        <x:v>定义POST /api/generation/jobs/{jobId}/downloads契约</x:v>
       </x:c>
       <x:c r="H134" s="13" t="str">
-        <x:v>共享Schema、类型和示例</x:v>
+        <x:v>variantIds与单一size共享Schema</x:v>
       </x:c>
       <x:c r="I134" s="13" t="str">
-        <x:v>合法与非法样例可被自动校验</x:v>
+        <x:v>合法与非法请求可自动校验</x:v>
       </x:c>
       <x:c r="J134" s="13" t="str">
         <x:v>—</x:v>
       </x:c>
       <x:c r="K134" s="13" t="str">
-        <x:v>待完成</x:v>
+        <x:v>已完成</x:v>
       </x:c>
       <x:c r="L134" s="13" t="str">
         <x:v>09-07～09-09</x:v>
       </x:c>
       <x:c r="M134" s="13" t="str">
-        <x:v>—</x:v>
+        <x:v>2026-08-21</x:v>
       </x:c>
       <x:c r="N134" s="13" t="str">
         <x:v>job/variant/asset UUID；archive_id UUID；归档键=用户+选择集+尺寸</x:v>
@@ -22553,25 +22553,25 @@
         <x:v>后端</x:v>
       </x:c>
       <x:c r="G135" s="13" t="str">
-        <x:v>实现POST/GET downloads输入校验</x:v>
+        <x:v>校验ZIP下载请求</x:v>
       </x:c>
       <x:c r="H135" s="13" t="str">
-        <x:v>边界校验与字段规范化</x:v>
+        <x:v>jobId、非空去重variantIds和允许size</x:v>
       </x:c>
       <x:c r="I135" s="13" t="str">
-        <x:v>非法输入在副作用前返回稳定400错误</x:v>
+        <x:v>无效输入在读取资产前返回稳定400错误</x:v>
       </x:c>
       <x:c r="J135" s="13" t="str">
         <x:v>BE-ARCHIVE-01</x:v>
       </x:c>
       <x:c r="K135" s="13" t="str">
-        <x:v>待完成</x:v>
+        <x:v>已完成</x:v>
       </x:c>
       <x:c r="L135" s="13" t="str">
         <x:v>09-07～09-09</x:v>
       </x:c>
       <x:c r="M135" s="13" t="str">
-        <x:v>—</x:v>
+        <x:v>2026-08-21</x:v>
       </x:c>
       <x:c r="N135" s="13" t="str">
         <x:v>job/variant/asset UUID；archive_id UUID；归档键=用户+选择集+尺寸</x:v>
@@ -22609,25 +22609,25 @@
         <x:v>后端</x:v>
       </x:c>
       <x:c r="G136" s="13" t="str">
-        <x:v>实现POST/GET downloads身份与权限校验</x:v>
+        <x:v>校验下载身份</x:v>
       </x:c>
       <x:c r="H136" s="13" t="str">
-        <x:v>服务端鉴权和所有权检查</x:v>
+        <x:v>当前服务端会话</x:v>
       </x:c>
       <x:c r="I136" s="13" t="str">
-        <x:v>未登录401；越权按规则403或404</x:v>
+        <x:v>未登录返回401</x:v>
       </x:c>
       <x:c r="J136" s="13" t="str">
         <x:v>BE-ARCHIVE-01</x:v>
       </x:c>
       <x:c r="K136" s="13" t="str">
-        <x:v>待完成</x:v>
+        <x:v>已完成</x:v>
       </x:c>
       <x:c r="L136" s="13" t="str">
         <x:v>09-07～09-09</x:v>
       </x:c>
       <x:c r="M136" s="13" t="str">
-        <x:v>—</x:v>
+        <x:v>2026-08-21</x:v>
       </x:c>
       <x:c r="N136" s="13" t="str">
         <x:v>job/variant/asset UUID；archive_id UUID；归档键=用户+选择集+尺寸</x:v>
@@ -22665,7 +22665,7 @@
         <x:v>后端</x:v>
       </x:c>
       <x:c r="G137" s="13" t="str">
-        <x:v>校验variantIds非空并去重</x:v>
+        <x:v>阻止空选择和重复ID</x:v>
       </x:c>
       <x:c r="H137" s="13" t="str">
         <x:v>选择集Schema</x:v>
@@ -22677,13 +22677,13 @@
         <x:v>—</x:v>
       </x:c>
       <x:c r="K137" s="13" t="str">
-        <x:v>待完成</x:v>
+        <x:v>已完成</x:v>
       </x:c>
       <x:c r="L137" s="13" t="str">
         <x:v>09-07～09-09</x:v>
       </x:c>
       <x:c r="M137" s="13" t="str">
-        <x:v>—</x:v>
+        <x:v>2026-08-21</x:v>
       </x:c>
       <x:c r="N137" s="13" t="str">
         <x:v>job/variant/asset UUID；archive_id UUID；归档键=用户+选择集+尺寸</x:v>
@@ -22721,25 +22721,25 @@
         <x:v>后端</x:v>
       </x:c>
       <x:c r="G138" s="13" t="str">
-        <x:v>校验所有variant属于本人</x:v>
+        <x:v>校验任务和所有方案归属</x:v>
       </x:c>
       <x:c r="H138" s="13" t="str">
-        <x:v>批量所有权检查</x:v>
+        <x:v>job→subject→variant所有权链</x:v>
       </x:c>
       <x:c r="I138" s="13" t="str">
-        <x:v>任一越权整请求失败</x:v>
+        <x:v>任一越权则整次请求失败</x:v>
       </x:c>
       <x:c r="J138" s="13" t="str">
         <x:v>—</x:v>
       </x:c>
       <x:c r="K138" s="13" t="str">
-        <x:v>待完成</x:v>
+        <x:v>已完成</x:v>
       </x:c>
       <x:c r="L138" s="13" t="str">
         <x:v>09-07～09-09</x:v>
       </x:c>
       <x:c r="M138" s="13" t="str">
-        <x:v>—</x:v>
+        <x:v>2026-08-21</x:v>
       </x:c>
       <x:c r="N138" s="13" t="str">
         <x:v>job/variant/asset UUID；archive_id UUID；归档键=用户+选择集+尺寸</x:v>
@@ -22780,22 +22780,22 @@
         <x:v>校验请求尺寸可用</x:v>
       </x:c>
       <x:c r="H139" s="13" t="str">
-        <x:v>asset size交集</x:v>
+        <x:v>每个variant必须存在同尺寸asset</x:v>
       </x:c>
       <x:c r="I139" s="13" t="str">
-        <x:v>缺失尺寸明确报错</x:v>
+        <x:v>任一缺失返回DOWNLOAD_NOT_READY</x:v>
       </x:c>
       <x:c r="J139" s="13" t="str">
         <x:v>—</x:v>
       </x:c>
       <x:c r="K139" s="13" t="str">
-        <x:v>待完成</x:v>
+        <x:v>已完成</x:v>
       </x:c>
       <x:c r="L139" s="13" t="str">
         <x:v>09-07～09-09</x:v>
       </x:c>
       <x:c r="M139" s="13" t="str">
-        <x:v>—</x:v>
+        <x:v>2026-08-21</x:v>
       </x:c>
       <x:c r="N139" s="13" t="str">
         <x:v>job/variant/asset UUID；archive_id UUID；归档键=用户+选择集+尺寸</x:v>
@@ -22833,25 +22833,25 @@
         <x:v>后端</x:v>
       </x:c>
       <x:c r="G140" s="13" t="str">
-        <x:v>计算稳定归档键</x:v>
+        <x:v>生成安全ZIP文件名</x:v>
       </x:c>
       <x:c r="H140" s="13" t="str">
-        <x:v>user+排序后variant+size hash</x:v>
+        <x:v>Bamboo任务ID和PNG文件名</x:v>
       </x:c>
       <x:c r="I140" s="13" t="str">
-        <x:v>相同选择24小时复用</x:v>
+        <x:v>文件名不接受客户端路径片段</x:v>
       </x:c>
       <x:c r="J140" s="13" t="str">
         <x:v>—</x:v>
       </x:c>
       <x:c r="K140" s="13" t="str">
-        <x:v>待完成</x:v>
+        <x:v>已完成</x:v>
       </x:c>
       <x:c r="L140" s="13" t="str">
         <x:v>09-07～09-09</x:v>
       </x:c>
       <x:c r="M140" s="13" t="str">
-        <x:v>—</x:v>
+        <x:v>2026-08-21</x:v>
       </x:c>
       <x:c r="N140" s="13" t="str">
         <x:v>job/variant/asset UUID；archive_id UUID；归档键=用户+选择集+尺寸</x:v>
@@ -22889,25 +22889,25 @@
         <x:v>后端</x:v>
       </x:c>
       <x:c r="G141" s="13" t="str">
-        <x:v>创建异步archive任务</x:v>
+        <x:v>在当前请求中创建ZIP</x:v>
       </x:c>
       <x:c r="H141" s="13" t="str">
-        <x:v>archive UUID和queued状态</x:v>
+        <x:v>一次请求一次归档</x:v>
       </x:c>
       <x:c r="I141" s="13" t="str">
-        <x:v>同键并发只创建一条</x:v>
+        <x:v>不建立当前需求未要求的异步归档任务</x:v>
       </x:c>
       <x:c r="J141" s="13" t="str">
         <x:v>—</x:v>
       </x:c>
       <x:c r="K141" s="13" t="str">
-        <x:v>待完成</x:v>
+        <x:v>已完成</x:v>
       </x:c>
       <x:c r="L141" s="13" t="str">
         <x:v>09-07～09-09</x:v>
       </x:c>
       <x:c r="M141" s="13" t="str">
-        <x:v>—</x:v>
+        <x:v>2026-08-21</x:v>
       </x:c>
       <x:c r="N141" s="13" t="str">
         <x:v>job/variant/asset UUID；archive_id UUID；归档键=用户+选择集+尺寸</x:v>
@@ -22945,25 +22945,25 @@
         <x:v>后端</x:v>
       </x:c>
       <x:c r="G142" s="13" t="str">
-        <x:v>按主体目录写PNG</x:v>
+        <x:v>读取私有PNG对象</x:v>
       </x:c>
       <x:c r="H142" s="13" t="str">
-        <x:v>slug/variant/size路径</x:v>
+        <x:v>Supabase Storage服务端下载</x:v>
       </x:c>
       <x:c r="I142" s="13" t="str">
-        <x:v>无路径穿越</x:v>
+        <x:v>不向其他用户暴露对象路径</x:v>
       </x:c>
       <x:c r="J142" s="13" t="str">
         <x:v>—</x:v>
       </x:c>
       <x:c r="K142" s="13" t="str">
-        <x:v>待完成</x:v>
+        <x:v>已完成</x:v>
       </x:c>
       <x:c r="L142" s="13" t="str">
         <x:v>09-07～09-09</x:v>
       </x:c>
       <x:c r="M142" s="13" t="str">
-        <x:v>—</x:v>
+        <x:v>2026-08-21</x:v>
       </x:c>
       <x:c r="N142" s="13" t="str">
         <x:v>job/variant/asset UUID；archive_id UUID；归档键=用户+选择集+尺寸</x:v>
@@ -23001,25 +23001,25 @@
         <x:v>后端</x:v>
       </x:c>
       <x:c r="G143" s="13" t="str">
-        <x:v>生成manifest.json</x:v>
+        <x:v>按主体和方案写入PNG</x:v>
       </x:c>
       <x:c r="H143" s="13" t="str">
-        <x:v>设置、版本、方案、尺寸、时间</x:v>
+        <x:v>subject-variant-slot-size.png</x:v>
       </x:c>
       <x:c r="I143" s="13" t="str">
-        <x:v>不含完整Prompt或密钥</x:v>
+        <x:v>同一ZIP内名称稳定且无路径穿越</x:v>
       </x:c>
       <x:c r="J143" s="13" t="str">
         <x:v>—</x:v>
       </x:c>
       <x:c r="K143" s="13" t="str">
-        <x:v>待完成</x:v>
+        <x:v>已完成</x:v>
       </x:c>
       <x:c r="L143" s="13" t="str">
         <x:v>09-07～09-09</x:v>
       </x:c>
       <x:c r="M143" s="13" t="str">
-        <x:v>—</x:v>
+        <x:v>2026-08-21</x:v>
       </x:c>
       <x:c r="N143" s="13" t="str">
         <x:v>job/variant/asset UUID；archive_id UUID；归档键=用户+选择集+尺寸</x:v>
@@ -23057,25 +23057,25 @@
         <x:v>后端</x:v>
       </x:c>
       <x:c r="G144" s="13" t="str">
-        <x:v>保存私有ZIP并标记ready</x:v>
+        <x:v>生成ZIP二进制响应</x:v>
       </x:c>
       <x:c r="H144" s="13" t="str">
-        <x:v>object path+expiresAt</x:v>
+        <x:v>application/zip</x:v>
       </x:c>
       <x:c r="I144" s="13" t="str">
-        <x:v>失败状态可重试</x:v>
+        <x:v>归档可被标准解压工具打开</x:v>
       </x:c>
       <x:c r="J144" s="13" t="str">
         <x:v>—</x:v>
       </x:c>
       <x:c r="K144" s="13" t="str">
-        <x:v>待完成</x:v>
+        <x:v>已完成</x:v>
       </x:c>
       <x:c r="L144" s="13" t="str">
         <x:v>09-07～09-09</x:v>
       </x:c>
       <x:c r="M144" s="13" t="str">
-        <x:v>—</x:v>
+        <x:v>2026-08-21</x:v>
       </x:c>
       <x:c r="N144" s="13" t="str">
         <x:v>job/variant/asset UUID；archive_id UUID；归档键=用户+选择集+尺寸</x:v>
@@ -23113,25 +23113,25 @@
         <x:v>后端</x:v>
       </x:c>
       <x:c r="G145" s="13" t="str">
-        <x:v>返回短时ZIP URL</x:v>
+        <x:v>设置私有不缓存响应</x:v>
       </x:c>
       <x:c r="H145" s="13" t="str">
-        <x:v>ready状态签名</x:v>
+        <x:v>private,no-store</x:v>
       </x:c>
       <x:c r="I145" s="13" t="str">
-        <x:v>24小时后归档和URL失效</x:v>
+        <x:v>浏览器或共享缓存不长期保存归档</x:v>
       </x:c>
       <x:c r="J145" s="13" t="str">
         <x:v>—</x:v>
       </x:c>
       <x:c r="K145" s="13" t="str">
-        <x:v>待完成</x:v>
+        <x:v>已完成</x:v>
       </x:c>
       <x:c r="L145" s="13" t="str">
         <x:v>09-07～09-09</x:v>
       </x:c>
       <x:c r="M145" s="13" t="str">
-        <x:v>—</x:v>
+        <x:v>2026-08-21</x:v>
       </x:c>
       <x:c r="N145" s="13" t="str">
         <x:v>job/variant/asset UUID；archive_id UUID；归档键=用户+选择集+尺寸</x:v>
@@ -23169,25 +23169,25 @@
         <x:v>后端</x:v>
       </x:c>
       <x:c r="G146" s="13" t="str">
-        <x:v>定义POST/GET downloads稳定错误码</x:v>
+        <x:v>返回下载文件名</x:v>
       </x:c>
       <x:c r="H146" s="13" t="str">
-        <x:v>错误枚举和HTTP映射</x:v>
+        <x:v>Content-Disposition attachment</x:v>
       </x:c>
       <x:c r="I146" s="13" t="str">
-        <x:v>前端无需解析内部错误正文</x:v>
+        <x:v>浏览器直接触发bamboo-icongen任务ZIP下载</x:v>
       </x:c>
       <x:c r="J146" s="13" t="str">
         <x:v>BE-ARCHIVE-02</x:v>
       </x:c>
       <x:c r="K146" s="13" t="str">
-        <x:v>待完成</x:v>
+        <x:v>已完成</x:v>
       </x:c>
       <x:c r="L146" s="13" t="str">
         <x:v>09-07～09-09</x:v>
       </x:c>
       <x:c r="M146" s="13" t="str">
-        <x:v>—</x:v>
+        <x:v>2026-08-21</x:v>
       </x:c>
       <x:c r="N146" s="13" t="str">
         <x:v>job/variant/asset UUID；archive_id UUID；归档键=用户+选择集+尺寸</x:v>
@@ -31509,7 +31509,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R0b26c508ae8c45fd"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R8d922f1b49544b2b"/>
   </x:tableParts>
 </x:worksheet>
 </file>
</xml_diff>

<commit_message>
feat: integrate library, favorites, auth and shared theme states
</commit_message>
<xml_diff>
--- a/outputs/2026-08-20-development-plan/IconGen-前后端原子级开发计划.xlsx
+++ b/outputs/2026-08-20-development-plan/IconGen-前后端原子级开发计划.xlsx
@@ -2,9 +2,9 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="阶段概览" sheetId="1" r:id="R760c11cde2174b81"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="前端开发计划" sheetId="2" r:id="R7b1e4804122f4fa2"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="后端开发计划" sheetId="3" r:id="R9c89e8b0ce424125"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="阶段概览" sheetId="1" r:id="Re0a106dcd00a45c9"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="前端开发计划" sheetId="2" r:id="R70ce9879f1144b36"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="后端开发计划" sheetId="3" r:id="Rcf131a6519ea41d9"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -444,7 +444,7 @@
   <x:sheetData>
     <x:row r="1" ht="36" customHeight="1">
       <x:c r="A1" s="2" t="str">
-        <x:v>Bamboo IconGen 原子级前后端开发计划</x:v>
+        <x:v>EASY DESIGN / ICON GEN 原子级前后端开发计划</x:v>
       </x:c>
       <x:c r="B1" s="2"/>
       <x:c r="C1" s="2"/>
@@ -596,7 +596,7 @@
   <x:sheetData>
     <x:row r="1" ht="34" customHeight="1">
       <x:c r="A1" s="7" t="str">
-        <x:v>Bamboo IconGen 前端原子级开发计划</x:v>
+        <x:v>EASY DESIGN / ICON GEN 前端原子级开发计划</x:v>
       </x:c>
       <x:c r="B1" s="7"/>
       <x:c r="C1" s="7"/>
@@ -1148,7 +1148,7 @@
         <x:v>建立首页和价格页路由与页面边界</x:v>
       </x:c>
       <x:c r="H12" s="13" t="str">
-        <x:v>首页、价格页、Bamboo IconGen 品牌导航和登录态导航</x:v>
+        <x:v>首页、价格页、EASY DESIGN / ICON GEN 品牌导航和登录态导航</x:v>
       </x:c>
       <x:c r="I12" s="13" t="str">
         <x:v>公开页可访问；访客不展示创建图标；登录态展示图标生成、我的图标和用户菜单</x:v>
@@ -15085,7 +15085,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R3e3635cbdb9e4703"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R0c5a645a02ae4aa8"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -15116,7 +15116,7 @@
   <x:sheetData>
     <x:row r="1" ht="34" customHeight="1">
       <x:c r="A1" s="7" t="str">
-        <x:v>Bamboo IconGen 后端原子级开发计划</x:v>
+        <x:v>EASY DESIGN / ICON GEN 后端原子级开发计划</x:v>
       </x:c>
       <x:c r="B1" s="7"/>
       <x:c r="C1" s="7"/>
@@ -22836,7 +22836,7 @@
         <x:v>生成安全ZIP文件名</x:v>
       </x:c>
       <x:c r="H140" s="13" t="str">
-        <x:v>Bamboo任务ID和PNG文件名</x:v>
+        <x:v>EASY DESIGN / ICON GEN任务ID和PNG文件名</x:v>
       </x:c>
       <x:c r="I140" s="13" t="str">
         <x:v>文件名不接受客户端路径片段</x:v>
@@ -23175,7 +23175,7 @@
         <x:v>Content-Disposition attachment</x:v>
       </x:c>
       <x:c r="I146" s="13" t="str">
-        <x:v>浏览器直接触发bamboo-icongen任务ZIP下载</x:v>
+        <x:v>浏览器直接触发easy-design任务ZIP下载</x:v>
       </x:c>
       <x:c r="J146" s="13" t="str">
         <x:v>BE-ARCHIVE-02</x:v>
@@ -30564,7 +30564,7 @@
         <x:v>注册或确定正式域名</x:v>
       </x:c>
       <x:c r="H278" t="str">
-        <x:v>Bamboo IconGen域名与注册商账号</x:v>
+        <x:v>EASY DESIGN / ICON GEN域名与注册商账号</x:v>
       </x:c>
       <x:c r="I278" t="str">
         <x:v>域名归项目方控制且可管理DNS</x:v>
@@ -31509,7 +31509,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R8d922f1b49544b2b"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Ra6f0059f2dac4a34"/>
   </x:tableParts>
 </x:worksheet>
 </file>
</xml_diff>